<commit_message>
Updates to excel file
</commit_message>
<xml_diff>
--- a/support materials/menuManager.xlsx
+++ b/support materials/menuManager.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hedbe\Dropbox\Papers\Paper.QEDs\Apps\plannerApp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hedbergec/Dropbox/Papers/Paper.QEDs/Apps/plannerApp/support materials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D7EA79D-AB9A-4D58-883A-C6113842A624}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A345039D-CD34-BE4A-A885-72353A9E3BDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3615" yWindow="3615" windowWidth="16875" windowHeight="10643" tabRatio="716" activeTab="6" xr2:uid="{8D89E9AD-B3C8-4CE6-A909-5B9DBA95DCBB}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16260" tabRatio="716" activeTab="7" xr2:uid="{8D89E9AD-B3C8-4CE6-A909-5B9DBA95DCBB}"/>
   </bookViews>
   <sheets>
     <sheet name="readme" sheetId="11" r:id="rId1"/>
@@ -149,7 +149,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="164">
   <si>
     <t>sample</t>
   </si>
@@ -307,21 +307,9 @@
     <t>Number covariates</t>
   </si>
   <si>
-    <t>Q2</t>
-  </si>
-  <si>
     <t>Covariate-treatment effect correlation (squared)</t>
   </si>
   <si>
-    <t>tau2</t>
-  </si>
-  <si>
-    <t>Variance of treatment effects across blocks</t>
-  </si>
-  <si>
-    <t>Variance of treatment effects across clusters</t>
-  </si>
-  <si>
     <t>Variance of treatment effects across longitudinal units</t>
   </si>
   <si>
@@ -346,9 +334,6 @@
     <t>p &lt;- nt/(nt+nc)</t>
   </si>
   <si>
-    <t>V &lt;- (nt+nc)*p*(1-p)</t>
-  </si>
-  <si>
     <t>srs_fixed_covariate_N</t>
   </si>
   <si>
@@ -361,9 +346,6 @@
     <t>srs_fixed_covariate_V</t>
   </si>
   <si>
-    <t>V &lt;- (nt+nc)*p*(1-p)*(1/(1-R2_1))</t>
-  </si>
-  <si>
     <t>blocked_fixed_nocovariate_N</t>
   </si>
   <si>
@@ -373,66 +355,36 @@
     <t>blocked_fixed_nocovariate_df</t>
   </si>
   <si>
-    <t>df &lt;- N-2*m</t>
-  </si>
-  <si>
     <t>blocked_fixed_nocovariate_V</t>
   </si>
   <si>
-    <t>iccbar &lt;- 1-icc</t>
-  </si>
-  <si>
-    <t>nbar &lt;- 2/(1/nt+1/nc)</t>
-  </si>
-  <si>
-    <t>V &lt;- 1/((iccbar+nbar*iccbar*(nc+nt))/(m*nc*nt))</t>
-  </si>
-  <si>
     <t>blocked_fixed_covariate_N</t>
   </si>
   <si>
     <t>blocked_fixed_covariate_df</t>
   </si>
   <si>
-    <t>df &lt;- N-2*m-q</t>
-  </si>
-  <si>
     <t>blocked_fixed_covariate_V</t>
   </si>
   <si>
-    <t>V &lt;-1/(((1-R2_1)*iccbar+nbar*iccbar*(nc+nt))/(m*nc*nt))</t>
-  </si>
-  <si>
     <t>blocked_random_nocovariate_N</t>
   </si>
   <si>
     <t>blocked_random_nocovariate_df</t>
   </si>
   <si>
-    <t>df &lt;- result &lt;- nbar*m - 2</t>
-  </si>
-  <si>
     <t>blocked_random_nocovariate_V</t>
   </si>
   <si>
-    <t>V &lt;- 1/((iccbar+nbar*tau2*(nc+nt))/(m*nc*nt))</t>
-  </si>
-  <si>
     <t>blocked_random_covariate_N</t>
   </si>
   <si>
     <t>blocked_random_covariate_df</t>
   </si>
   <si>
-    <t>df &lt;- result &lt;- nbar*m - 2 - q</t>
-  </si>
-  <si>
     <t>blocked_random_covariate_V</t>
   </si>
   <si>
-    <t>V &lt;- 1/(((1-R2_1)*iccbar+(1-Q2)*nbar*tau2*iccbar*(nc+nt))/(m*nc*nt))</t>
-  </si>
-  <si>
     <t>clustered_random_nocovariate_N</t>
   </si>
   <si>
@@ -451,27 +403,15 @@
     <t>p &lt;- mt/(mt+mc)</t>
   </si>
   <si>
-    <t>de &lt;- 1+(n-1)*icc</t>
-  </si>
-  <si>
-    <t>V &lt;- 1/(de/(p*(1-p)*(mt+mc)*n))</t>
-  </si>
-  <si>
     <t>clustered_random_covariate_N</t>
   </si>
   <si>
     <t>clustered_random_covariate_df</t>
   </si>
   <si>
-    <t>mt + mc - 2 - q</t>
-  </si>
-  <si>
     <t>clustered_random_covariate_V</t>
   </si>
   <si>
-    <t>de &lt;- 1+(n-1)*icc-(R2_1+(n*R2_2-R2_1)*icc)</t>
-  </si>
-  <si>
     <t>its_fixed_nocovariate_N</t>
   </si>
   <si>
@@ -589,9 +529,6 @@
     <t>Variance reduction in outcome (individuals)</t>
   </si>
   <si>
-    <t>Variance reduction in outcome (blocks)</t>
-  </si>
-  <si>
     <t>Number of  clusters</t>
   </si>
   <si>
@@ -656,22 +593,63 @@
   </si>
   <si>
     <t>Difference in Differences (DiD)</t>
+  </si>
+  <si>
+    <t>Ratio of Variance of treatment effects across blocks to variance of means across blocks</t>
+  </si>
+  <si>
+    <t>upsilon</t>
+  </si>
+  <si>
+    <t>n &lt;- nt+nc</t>
+  </si>
+  <si>
+    <t>V &lt;- n*p*(1-p)*(1/(1-R2_1))</t>
+  </si>
+  <si>
+    <t>V &lt;- n*p*(1-p)</t>
+  </si>
+  <si>
+    <t>m &lt;- mt+mc</t>
+  </si>
+  <si>
+    <t>df &lt;- mt + mc - 2 - q</t>
+  </si>
+  <si>
+    <t>#From appendix in DiD Chapter</t>
+  </si>
+  <si>
+    <t>df &lt;- m*(nt+nc)-2</t>
+  </si>
+  <si>
+    <t>df &lt;- m*(nt+nc)-2-q</t>
+  </si>
+  <si>
+    <t>V &lt;- m*n*p*(1-p)*(1/(1+(n-1)*icc))</t>
+  </si>
+  <si>
+    <t>V &lt;- m*n*p*(1-p)*(1/(1+(n-1)*icc-(R2_1+(n*R2_2-R2_1)*icc)))</t>
+  </si>
+  <si>
+    <t>V &lt;- m*n*p*(1-p)*(1/(1+(n*p*(1-p)*upsilon)*icc-(R2_1+(n*p*(1-p)*upsilon)*R2_2-R2_1)*icc))</t>
+  </si>
+  <si>
+    <t>V &lt;- m*n*p*(1-p)*(1/(1+(n*p*(1-p)*upsilon)*icc))</t>
+  </si>
+  <si>
+    <t>V &lt;- m*n*p*(1-p)*(1/(1-icc))</t>
+  </si>
+  <si>
+    <t>V &lt;- m*n*p*(1-p)*(1/((1-icc)-(R2_1-R2_1*icc)))</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -691,6 +669,17 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -712,24 +701,206 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="10">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Consolas"/>
+        <family val="3"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Consolas"/>
+        <family val="3"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Consolas"/>
+        <family val="3"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Consolas"/>
+        <family val="3"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Consolas"/>
+        <family val="3"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Consolas"/>
+        <family val="3"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Consolas"/>
+        <family val="3"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Consolas"/>
+        <family val="3"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -746,6 +917,18 @@
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <person displayName="E. C. Hedberg" id="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" userId="2a678a435b491d97" providerId="Windows Live"/>
 </personList>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6152DF64-9A11-42D3-B695-178EF7A61CD5}" name="Table3" displayName="Table3" ref="A1:D34" headerRowCount="0" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{14FCBBA3-4721-4280-B533-C0FC542668AA}" name="Column1" headerRowDxfId="7" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{E90FB251-9DD0-40B0-A06B-487DE170DB7D}" name="Column2" headerRowDxfId="5" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{1DDFB4AE-3D35-415F-AC9F-F95F752C46CF}" name="Column3" headerRowDxfId="3" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{5BDFB90D-F447-456A-9633-044179DB9760}" name="Column4" headerRowDxfId="1" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="1"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1086,93 +1269,93 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C51C3392-495A-4716-B7D0-8CB1570246E2}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A3" s="3" t="str">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="str">
         <f>HYPERLINK(sample!A1)</f>
         <v>sample</v>
       </c>
       <c r="B3" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A4" s="3" t="str">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="str">
         <f>HYPERLINK(design!A1)</f>
         <v>design</v>
       </c>
       <c r="B4" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A5" s="3" t="str">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="str">
         <f>HYPERLINK(inference!A1)</f>
         <v>inference</v>
       </c>
       <c r="B5" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A6" s="3" t="str">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="str">
         <f>HYPERLINK(model!A1)</f>
         <v>model</v>
       </c>
       <c r="B6" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A7" s="3" t="str">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="str">
         <f>HYPERLINK(stat!A1)</f>
         <v>stat</v>
       </c>
       <c r="B7" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A8" s="3" t="str">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="str">
         <f>HYPERLINK(input!A1)</f>
         <v>input</v>
       </c>
       <c r="B8" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A9" s="3"/>
+        <v>110</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="2"/>
       <c r="C9" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A10" s="3" t="str">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="str">
         <f>HYPERLINK(code!A1,"code")</f>
         <v>code</v>
       </c>
       <c r="B10" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="C11" t="s">
-        <v>128</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -1183,9 +1366,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A96E0447-8401-42C5-BE02-401F505AE938}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1193,7 +1376,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1201,7 +1384,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1217,12 +1400,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62AA0D0E-E4D1-469A-AF1F-085E17D5518F}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="29.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -1236,67 +1419,67 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>133</v>
+        <v>113</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>131</v>
+        <v>111</v>
       </c>
       <c r="C3" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>132</v>
+        <v>112</v>
       </c>
       <c r="C4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>166</v>
+        <v>145</v>
       </c>
       <c r="D5" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>167</v>
+        <v>146</v>
       </c>
       <c r="D6" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>113</v>
+        <v>93</v>
       </c>
       <c r="B7" t="s">
-        <v>168</v>
+        <v>147</v>
       </c>
       <c r="D7" t="b">
         <v>1</v>
@@ -1310,13 +1493,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33C6AD60-7AB8-4CAF-9726-0F1707E818DE}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.1328125" customWidth="1"/>
+    <col min="3" max="3" width="5.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -1339,10 +1522,10 @@
         <v>11</v>
       </c>
       <c r="H1" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -1365,7 +1548,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1387,14 +1570,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F39838A5-C062-40CB-BD39-4466E5E1974A}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.1328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="5.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -1417,15 +1600,15 @@
         <v>11</v>
       </c>
       <c r="H1" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>134</v>
+        <v>114</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
@@ -1446,12 +1629,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>135</v>
+        <v>115</v>
       </c>
       <c r="C3" t="b">
         <v>1</v>
@@ -1471,13 +1654,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9306200-6D5D-404E-9AA4-2D83AC7E89FD}">
   <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="22.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>20</v>
       </c>
@@ -1500,10 +1683,10 @@
         <v>11</v>
       </c>
       <c r="H1" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -1529,7 +1712,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -1555,7 +1738,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -1589,8 +1772,8 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7085B87C-0BDF-4509-A80F-252767BE3B26}">
-  <dimension ref="A1:X16"/>
-  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:X15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" style="1" customWidth="1"/>
@@ -1598,19 +1781,19 @@
     <col min="4" max="4" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="5.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="5.33203125" style="1" customWidth="1"/>
-    <col min="8" max="9" width="7.796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="7.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.1328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="7.796875" style="1" customWidth="1"/>
-    <col min="15" max="16" width="9.1328125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="9.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="7.83203125" style="1" customWidth="1"/>
+    <col min="15" max="16" width="9.1640625" style="1" customWidth="1"/>
     <col min="17" max="17" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="14.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="19" max="21" width="49.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="22" max="23" width="55.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="16384" width="9.1328125" style="1"/>
+    <col min="24" max="16384" width="9.1640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>27</v>
       </c>
@@ -1630,7 +1813,7 @@
         <v>11</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>113</v>
+        <v>93</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>13</v>
@@ -1681,10 +1864,10 @@
         <v>36</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.45">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>37</v>
       </c>
@@ -1729,19 +1912,19 @@
         <v>c(4,40)</v>
       </c>
       <c r="T2" s="1" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="U2" s="1" t="s">
-        <v>147</v>
+        <v>126</v>
       </c>
       <c r="V2" s="1" t="s">
-        <v>161</v>
+        <v>140</v>
       </c>
       <c r="W2" s="1" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.45">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>38</v>
       </c>
@@ -1782,23 +1965,23 @@
         <v>5</v>
       </c>
       <c r="R3" s="1" t="str">
-        <f t="shared" ref="R3:R16" si="0">_xlfn.CONCAT("c(",O3,",",P3,")")</f>
+        <f t="shared" ref="R3:R15" si="0">_xlfn.CONCAT("c(",O3,",",P3,")")</f>
         <v>c(2,40)</v>
       </c>
       <c r="T3" s="1" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="U3" s="1" t="s">
-        <v>148</v>
+        <v>127</v>
       </c>
       <c r="V3" s="1" t="s">
-        <v>136</v>
+        <v>116</v>
       </c>
       <c r="W3" s="1" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.45">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>39</v>
       </c>
@@ -1843,19 +2026,19 @@
         <v>c(2,40)</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="U4" s="1" t="s">
-        <v>149</v>
+        <v>128</v>
       </c>
       <c r="V4" s="1" t="s">
-        <v>137</v>
+        <v>117</v>
       </c>
       <c r="W4" s="1" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.45">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>40</v>
       </c>
@@ -1897,19 +2080,19 @@
         <v>c(4,150)</v>
       </c>
       <c r="T5" s="1" t="s">
-        <v>151</v>
+        <v>130</v>
       </c>
       <c r="U5" s="1" t="s">
-        <v>150</v>
+        <v>129</v>
       </c>
       <c r="V5" s="1" t="s">
-        <v>162</v>
+        <v>141</v>
       </c>
       <c r="W5" s="1" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.45">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>41</v>
       </c>
@@ -1957,25 +2140,25 @@
         <v>c(2,150)</v>
       </c>
       <c r="S6" s="1" t="s">
-        <v>138</v>
+        <v>118</v>
       </c>
       <c r="T6" s="1" t="s">
-        <v>153</v>
+        <v>132</v>
       </c>
       <c r="U6" s="1" t="s">
-        <v>154</v>
+        <v>133</v>
       </c>
       <c r="V6" s="1" t="s">
-        <v>163</v>
+        <v>142</v>
       </c>
       <c r="W6" s="1" t="s">
-        <v>163</v>
+        <v>142</v>
       </c>
       <c r="X6" s="1" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.45">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>42</v>
       </c>
@@ -2023,25 +2206,25 @@
         <v>c(2,150)</v>
       </c>
       <c r="S7" s="1" t="s">
-        <v>139</v>
+        <v>119</v>
       </c>
       <c r="T7" s="1" t="s">
-        <v>152</v>
+        <v>131</v>
       </c>
       <c r="U7" s="1" t="s">
-        <v>155</v>
+        <v>134</v>
       </c>
       <c r="V7" s="1" t="s">
-        <v>164</v>
+        <v>143</v>
       </c>
       <c r="W7" s="1" t="s">
-        <v>164</v>
+        <v>143</v>
       </c>
       <c r="X7" s="1" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.45">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>43</v>
       </c>
@@ -2087,19 +2270,19 @@
         <v>c(2,100)</v>
       </c>
       <c r="T8" s="1" t="s">
-        <v>156</v>
+        <v>135</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>156</v>
+        <v>135</v>
       </c>
       <c r="V8" s="1" t="s">
-        <v>156</v>
+        <v>135</v>
       </c>
       <c r="W8" s="1" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.45">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>44</v>
       </c>
@@ -2145,19 +2328,19 @@
         <v>c(2,100)</v>
       </c>
       <c r="T9" s="1" t="s">
-        <v>157</v>
+        <v>136</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>157</v>
+        <v>136</v>
       </c>
       <c r="V9" s="1" t="s">
-        <v>157</v>
+        <v>136</v>
       </c>
       <c r="W9" s="1" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.45">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>45</v>
       </c>
@@ -2202,19 +2385,19 @@
         <v>c(0.01,0.2)</v>
       </c>
       <c r="T10" s="1" t="s">
-        <v>144</v>
+        <v>124</v>
       </c>
       <c r="U10" s="1" t="s">
-        <v>144</v>
+        <v>124</v>
       </c>
       <c r="V10" s="1" t="s">
-        <v>144</v>
+        <v>124</v>
       </c>
       <c r="W10" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.45">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>46</v>
       </c>
@@ -2253,24 +2436,27 @@
         <v>c(0,0.99)</v>
       </c>
       <c r="S11" s="1" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="T11" s="1" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="U11" s="1" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="V11" s="1" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="W11" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.45">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>47</v>
+      </c>
+      <c r="C12" s="1" t="b">
+        <v>1</v>
       </c>
       <c r="D12" s="1" t="b">
         <v>1</v>
@@ -2298,19 +2484,19 @@
         <v>c(0,0.99)</v>
       </c>
       <c r="T12" s="1" t="s">
-        <v>146</v>
+        <v>52</v>
       </c>
       <c r="U12" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="V12" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="W12" s="4" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.45">
+        <v>137</v>
+      </c>
+      <c r="V12" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="W12" s="3" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>48</v>
       </c>
@@ -2364,10 +2550,10 @@
         <v>49</v>
       </c>
       <c r="X13" s="1" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.45">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>50</v>
       </c>
@@ -2412,21 +2598,21 @@
         <v>51</v>
       </c>
       <c r="T14" s="1" t="s">
-        <v>160</v>
+        <v>139</v>
       </c>
       <c r="U14" s="1" t="s">
-        <v>160</v>
+        <v>139</v>
       </c>
       <c r="V14" s="1" t="s">
-        <v>160</v>
+        <v>139</v>
       </c>
       <c r="W14" s="1" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.45">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>52</v>
+        <v>149</v>
       </c>
       <c r="C15" s="1" t="b">
         <v>1</v>
@@ -2434,6 +2620,9 @@
       <c r="I15" s="1" t="b">
         <v>1</v>
       </c>
+      <c r="J15" s="1" t="b">
+        <v>1</v>
+      </c>
       <c r="K15" s="1" t="b">
         <v>1</v>
       </c>
@@ -2441,74 +2630,26 @@
         <v>1</v>
       </c>
       <c r="O15" s="1">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="P15" s="1">
-        <v>0.99</v>
+        <v>3.25</v>
       </c>
       <c r="Q15" s="1">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="R15" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>c(0,0.99)</v>
+        <v>c(0.01,3.25)</v>
       </c>
       <c r="T15" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="U15" s="1" t="s">
-        <v>53</v>
+        <v>148</v>
       </c>
       <c r="V15" s="1" t="s">
         <v>53</v>
       </c>
       <c r="W15" s="1" t="s">
         <v>53</v>
-      </c>
-    </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.45">
-      <c r="A16" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C16" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="I16" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="J16" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="K16" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="N16" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O16" s="1">
-        <v>0</v>
-      </c>
-      <c r="P16" s="1">
-        <v>3.25</v>
-      </c>
-      <c r="Q16" s="1">
-        <v>0.15</v>
-      </c>
-      <c r="R16" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>c(0,3.25)</v>
-      </c>
-      <c r="T16" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="U16" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="V16" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="W16" s="1" t="s">
-        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -2520,351 +2661,324 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D24D9501-1928-C24A-A5F8-EF63F20DDAEF}">
-  <dimension ref="A1:D44"/>
-  <sheetFormatPr defaultColWidth="11.33203125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:D34"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.33203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="33.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="42.1640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5" style="5" customWidth="1"/>
+    <col min="4" max="4" width="84.6640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="11.33203125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A2" s="2" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B4" s="5" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A3" s="2" t="s">
+      <c r="C4" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B5" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="4" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A4" s="2" t="s">
+      <c r="B6" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="B4" t="s">
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="C4" t="s">
+      <c r="B7" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A5" s="2" t="s">
+      <c r="B8" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A6" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B6" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A7" s="2" t="s">
+      <c r="C10" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B7" t="s">
-        <v>64</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="B11" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" s="4" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A8" s="2" t="s">
+      <c r="B12" s="5" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B13" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" s="4" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A9" s="2" t="s">
+      <c r="B14" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B9" t="s">
-        <v>72</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="B15" s="5" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" s="4" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A10" s="2" t="s">
+      <c r="B16" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B17" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="C10" t="s">
+      <c r="B18" s="5" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="D10" t="s">
+      <c r="B19" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" s="4" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A11" s="2" t="s">
+      <c r="B20" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="B11" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A12" s="2" t="s">
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B12" t="s">
-        <v>72</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="B21" s="5" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A13" s="2" t="s">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B13" t="s">
-        <v>76</v>
-      </c>
-      <c r="C13" t="s">
-        <v>77</v>
-      </c>
-      <c r="D13" t="s">
+      <c r="B22" s="5" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A14" s="2" t="s">
+      <c r="C22" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="B14" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A15" s="2" t="s">
+      <c r="B23" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="B15" t="s">
-        <v>77</v>
-      </c>
-      <c r="C15" t="s">
+      <c r="B24" s="5" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" s="4" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A16" s="2" t="s">
+      <c r="B25" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A27" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A28" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A29" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B16" t="s">
-        <v>76</v>
-      </c>
-      <c r="C16" t="s">
-        <v>77</v>
-      </c>
-      <c r="D16" t="s">
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A30" s="4" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A17" s="2" t="s">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="B17" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A18" s="2" t="s">
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B18" t="s">
-        <v>77</v>
-      </c>
-      <c r="C18" t="s">
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" s="4" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A19" s="2" t="s">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="B19" t="s">
-        <v>76</v>
-      </c>
-      <c r="C19" t="s">
-        <v>77</v>
-      </c>
-      <c r="D19" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A20" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="B20" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A21" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B21" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A22" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="B22" t="s">
-        <v>99</v>
-      </c>
-      <c r="C22" t="s">
-        <v>100</v>
-      </c>
-      <c r="D22" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A23" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="B23" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A24" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="B24" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A25" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="B25" t="s">
-        <v>99</v>
-      </c>
-      <c r="C25" t="s">
-        <v>106</v>
-      </c>
-      <c r="D25" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A26" s="2" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A27" s="2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A28" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A29" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A30" s="2" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A31" s="2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A32" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="B32" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A33" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="B33" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A34" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="B34" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A35" s="2"/>
-    </row>
-    <row r="36" spans="1:2" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A36" s="2"/>
-    </row>
-    <row r="37" spans="1:2" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A37" s="2"/>
-    </row>
-    <row r="38" spans="1:2" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A38" s="2"/>
-    </row>
-    <row r="39" spans="1:2" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A39" s="2"/>
-    </row>
-    <row r="40" spans="1:2" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A40" s="2"/>
-    </row>
-    <row r="41" spans="1:2" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A41" s="2"/>
-    </row>
-    <row r="42" spans="1:2" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A42" s="2"/>
-    </row>
-    <row r="43" spans="1:2" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A43" s="2"/>
-    </row>
-    <row r="44" spans="1:2" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A44" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
+  <tableParts count="1">
+    <tablePart r:id="rId3"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix steps in sliders, qed data
</commit_message>
<xml_diff>
--- a/support materials/menuManager.xlsx
+++ b/support materials/menuManager.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hedbergec/Dropbox/Papers/Paper.QEDs/Apps/plannerApp/support materials/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hedbe\Dropbox\Papers\Paper.QEDs\Apps\plannerApp\support materials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A345039D-CD34-BE4A-A885-72353A9E3BDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD618F96-4680-4A44-8044-8EA83821097A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16260" tabRatio="716" activeTab="7" xr2:uid="{8D89E9AD-B3C8-4CE6-A909-5B9DBA95DCBB}"/>
+    <workbookView xWindow="31350" yWindow="1515" windowWidth="21600" windowHeight="11145" tabRatio="716" activeTab="6" xr2:uid="{8D89E9AD-B3C8-4CE6-A909-5B9DBA95DCBB}"/>
   </bookViews>
   <sheets>
     <sheet name="readme" sheetId="11" r:id="rId1"/>
@@ -52,6 +52,7 @@
     <author>tc={53AAC73E-37CD-4F93-952F-58532973ACC7}</author>
     <author>tc={404E6D2E-D072-435D-810D-184FE609405B}</author>
     <author>tc={1DE218DE-31C8-4B3E-95DD-574166043541}</author>
+    <author>tc={CA4BCEC2-9B3E-4FC5-B2C2-41BB34B83579}</author>
   </authors>
   <commentList>
     <comment ref="G1" authorId="0" shapeId="0" xr:uid="{0713FE03-72D3-4E97-9C1A-4F35BCE26CD6}">
@@ -126,6 +127,14 @@
     Not used yet, but made with excel formula</t>
       </text>
     </comment>
+    <comment ref="T1" authorId="9" shapeId="0" xr:uid="{CA4BCEC2-9B3E-4FC5-B2C2-41BB34B83579}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not used yet, but made with excel formula</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -149,7 +158,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="166">
   <si>
     <t>sample</t>
   </si>
@@ -641,13 +650,19 @@
   </si>
   <si>
     <t>V &lt;- m*n*p*(1-p)*(1/((1-icc)-(R2_1-R2_1*icc)))</t>
+  </si>
+  <si>
+    <t>ui_step_range</t>
+  </si>
+  <si>
+    <t>ui_step_exact</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -680,6 +695,12 @@
       <sz val="11"/>
       <name val="Consolas"/>
       <family val="3"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1255,6 +1276,9 @@
   <threadedComment ref="R1" dT="2021-07-10T00:53:30.43" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{1DE218DE-31C8-4B3E-95DD-574166043541}">
     <text>Not used yet, but made with excel formula</text>
   </threadedComment>
+  <threadedComment ref="T1" dT="2021-07-10T00:53:30.43" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{CA4BCEC2-9B3E-4FC5-B2C2-41BB34B83579}">
+    <text>Not used yet, but made with excel formula</text>
+  </threadedComment>
 </ThreadedComments>
 </file>
 
@@ -1269,22 +1293,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C51C3392-495A-4716-B7D0-8CB1570246E2}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.6640625" customWidth="1"/>
+    <col min="1" max="1" width="21.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="str">
         <f>HYPERLINK(sample!A1)</f>
         <v>sample</v>
@@ -1293,7 +1317,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="str">
         <f>HYPERLINK(design!A1)</f>
         <v>design</v>
@@ -1302,7 +1326,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="str">
         <f>HYPERLINK(inference!A1)</f>
         <v>inference</v>
@@ -1311,7 +1335,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="str">
         <f>HYPERLINK(model!A1)</f>
         <v>model</v>
@@ -1320,7 +1344,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="str">
         <f>HYPERLINK(stat!A1)</f>
         <v>stat</v>
@@ -1329,7 +1353,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="str">
         <f>HYPERLINK(input!A1)</f>
         <v>input</v>
@@ -1338,13 +1362,13 @@
         <v>110</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="C9" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="str">
         <f>HYPERLINK(code!A1,"code")</f>
         <v>code</v>
@@ -1353,7 +1377,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
         <v>108</v>
       </c>
@@ -1366,9 +1390,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A96E0447-8401-42C5-BE02-401F505AE938}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1376,7 +1400,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1384,7 +1408,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1400,12 +1424,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62AA0D0E-E4D1-469A-AF1F-085E17D5518F}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -1419,7 +1443,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1430,7 +1454,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1441,7 +1465,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1452,7 +1476,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -1463,7 +1487,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -1474,7 +1498,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>93</v>
       </c>
@@ -1493,13 +1517,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33C6AD60-7AB8-4CAF-9726-0F1707E818DE}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.1640625" customWidth="1"/>
+    <col min="3" max="3" width="5.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -1525,7 +1549,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -1548,7 +1572,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1570,14 +1594,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F39838A5-C062-40CB-BD39-4466E5E1974A}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -1603,7 +1627,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -1629,7 +1653,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -1654,13 +1678,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9306200-6D5D-404E-9AA4-2D83AC7E89FD}">
   <dimension ref="A1:H4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>20</v>
       </c>
@@ -1686,7 +1710,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -1712,7 +1736,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -1738,7 +1762,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -1772,28 +1796,29 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7085B87C-0BDF-4509-A80F-252767BE3B26}">
-  <dimension ref="A1:X15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:Z15"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" style="1" customWidth="1"/>
     <col min="3" max="3" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="5.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.33203125" style="1" customWidth="1"/>
-    <col min="8" max="9" width="7.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="5.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.28515625" style="1" customWidth="1"/>
+    <col min="8" max="9" width="7.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="7.83203125" style="1" customWidth="1"/>
-    <col min="15" max="16" width="9.1640625" style="1" customWidth="1"/>
-    <col min="17" max="17" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="21" width="49.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="55.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="16384" width="9.1640625" style="1"/>
+    <col min="11" max="11" width="9.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="7.85546875" style="1" customWidth="1"/>
+    <col min="15" max="16" width="9.140625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="14.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="20" width="14.7109375" style="1" customWidth="1"/>
+    <col min="21" max="23" width="49.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="55.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>27</v>
       </c>
@@ -1849,25 +1874,31 @@
         <v>30</v>
       </c>
       <c r="S1" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="U1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>37</v>
       </c>
@@ -1911,20 +1942,26 @@
         <f>_xlfn.CONCAT("c(",O2,",",P2,")")</f>
         <v>c(4,40)</v>
       </c>
-      <c r="T2" s="1" t="s">
+      <c r="S2" s="1">
+        <v>1</v>
+      </c>
+      <c r="T2" s="1">
+        <v>1</v>
+      </c>
+      <c r="V2" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="U2" s="1" t="s">
+      <c r="W2" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="V2" s="1" t="s">
+      <c r="X2" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="W2" s="1" t="s">
+      <c r="Y2" s="1" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>38</v>
       </c>
@@ -1968,20 +2005,26 @@
         <f t="shared" ref="R3:R15" si="0">_xlfn.CONCAT("c(",O3,",",P3,")")</f>
         <v>c(2,40)</v>
       </c>
-      <c r="T3" s="1" t="s">
+      <c r="S3" s="1">
+        <v>1</v>
+      </c>
+      <c r="T3" s="1">
+        <v>1</v>
+      </c>
+      <c r="V3" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="U3" s="1" t="s">
+      <c r="W3" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="V3" s="1" t="s">
+      <c r="X3" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="W3" s="1" t="s">
+      <c r="Y3" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>39</v>
       </c>
@@ -2025,20 +2068,26 @@
         <f t="shared" si="0"/>
         <v>c(2,40)</v>
       </c>
-      <c r="T4" s="1" t="s">
+      <c r="S4" s="1">
+        <v>1</v>
+      </c>
+      <c r="T4" s="1">
+        <v>1</v>
+      </c>
+      <c r="V4" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="U4" s="1" t="s">
+      <c r="W4" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="V4" s="1" t="s">
+      <c r="X4" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="W4" s="1" t="s">
+      <c r="Y4" s="1" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>40</v>
       </c>
@@ -2079,20 +2128,26 @@
         <f t="shared" si="0"/>
         <v>c(4,150)</v>
       </c>
-      <c r="T5" s="1" t="s">
+      <c r="S5" s="1">
+        <v>1</v>
+      </c>
+      <c r="T5" s="1">
+        <v>1</v>
+      </c>
+      <c r="V5" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="U5" s="1" t="s">
+      <c r="W5" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="V5" s="1" t="s">
+      <c r="X5" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="W5" s="1" t="s">
+      <c r="Y5" s="1" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>41</v>
       </c>
@@ -2139,26 +2194,32 @@
         <f t="shared" si="0"/>
         <v>c(2,150)</v>
       </c>
-      <c r="S6" s="1" t="s">
+      <c r="S6" s="1">
+        <v>1</v>
+      </c>
+      <c r="T6" s="1">
+        <v>1</v>
+      </c>
+      <c r="U6" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="T6" s="1" t="s">
+      <c r="V6" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="U6" s="1" t="s">
+      <c r="W6" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="V6" s="1" t="s">
+      <c r="X6" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="W6" s="1" t="s">
+      <c r="Y6" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="X6" s="1" t="s">
+      <c r="Z6" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>42</v>
       </c>
@@ -2205,26 +2266,32 @@
         <f t="shared" si="0"/>
         <v>c(2,150)</v>
       </c>
-      <c r="S7" s="1" t="s">
+      <c r="S7" s="1">
+        <v>1</v>
+      </c>
+      <c r="T7" s="1">
+        <v>1</v>
+      </c>
+      <c r="U7" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="T7" s="1" t="s">
+      <c r="V7" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="U7" s="1" t="s">
+      <c r="W7" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="V7" s="1" t="s">
+      <c r="X7" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="W7" s="1" t="s">
+      <c r="Y7" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="X7" s="1" t="s">
+      <c r="Z7" s="1" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>43</v>
       </c>
@@ -2269,11 +2336,11 @@
         <f t="shared" si="0"/>
         <v>c(2,100)</v>
       </c>
-      <c r="T8" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="U8" s="1" t="s">
-        <v>135</v>
+      <c r="S8" s="1">
+        <v>1</v>
+      </c>
+      <c r="T8" s="1">
+        <v>1</v>
       </c>
       <c r="V8" s="1" t="s">
         <v>135</v>
@@ -2281,8 +2348,14 @@
       <c r="W8" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="X8" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="Y8" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>44</v>
       </c>
@@ -2327,11 +2400,11 @@
         <f t="shared" si="0"/>
         <v>c(2,100)</v>
       </c>
-      <c r="T9" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="U9" s="1" t="s">
-        <v>136</v>
+      <c r="S9" s="1">
+        <v>1</v>
+      </c>
+      <c r="T9" s="1">
+        <v>1</v>
       </c>
       <c r="V9" s="1" t="s">
         <v>136</v>
@@ -2339,8 +2412,14 @@
       <c r="W9" s="1" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="X9" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="Y9" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>45</v>
       </c>
@@ -2384,11 +2463,11 @@
         <f t="shared" si="0"/>
         <v>c(0.01,0.2)</v>
       </c>
-      <c r="T10" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="U10" s="1" t="s">
-        <v>124</v>
+      <c r="S10" s="1">
+        <v>0.01</v>
+      </c>
+      <c r="T10" s="1">
+        <v>0.01</v>
       </c>
       <c r="V10" s="1" t="s">
         <v>124</v>
@@ -2396,8 +2475,14 @@
       <c r="W10" s="1" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="X10" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="Y10" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>46</v>
       </c>
@@ -2435,14 +2520,14 @@
         <f t="shared" si="0"/>
         <v>c(0,0.99)</v>
       </c>
-      <c r="S11" s="1" t="s">
+      <c r="S11" s="1">
+        <v>0.01</v>
+      </c>
+      <c r="T11" s="1">
+        <v>0.01</v>
+      </c>
+      <c r="U11" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="T11" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="U11" s="1" t="s">
-        <v>125</v>
       </c>
       <c r="V11" s="1" t="s">
         <v>125</v>
@@ -2450,8 +2535,14 @@
       <c r="W11" s="1" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="X11" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="Y11" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>47</v>
       </c>
@@ -2483,20 +2574,26 @@
         <f t="shared" si="0"/>
         <v>c(0,0.99)</v>
       </c>
-      <c r="T12" s="1" t="s">
+      <c r="S12" s="1">
+        <v>0.01</v>
+      </c>
+      <c r="T12" s="1">
+        <v>0.01</v>
+      </c>
+      <c r="V12" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="U12" s="1" t="s">
+      <c r="W12" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="V12" s="3" t="s">
+      <c r="X12" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="W12" s="3" t="s">
+      <c r="Y12" s="3" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>48</v>
       </c>
@@ -2537,11 +2634,11 @@
         <f t="shared" si="0"/>
         <v>c(0,0.99)</v>
       </c>
-      <c r="T13" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="U13" s="1" t="s">
-        <v>49</v>
+      <c r="S13" s="1">
+        <v>0.01</v>
+      </c>
+      <c r="T13" s="1">
+        <v>0.01</v>
       </c>
       <c r="V13" s="1" t="s">
         <v>49</v>
@@ -2550,10 +2647,16 @@
         <v>49</v>
       </c>
       <c r="X13" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="Y13" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="Z13" s="1" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>50</v>
       </c>
@@ -2582,7 +2685,7 @@
         <v>1</v>
       </c>
       <c r="O14" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P14" s="1">
         <v>6</v>
@@ -2592,16 +2695,16 @@
       </c>
       <c r="R14" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>c(0,6)</v>
-      </c>
-      <c r="S14" s="1" t="s">
+        <v>c(1,6)</v>
+      </c>
+      <c r="S14" s="1">
+        <v>1</v>
+      </c>
+      <c r="T14" s="1">
+        <v>1</v>
+      </c>
+      <c r="U14" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="T14" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="U14" s="1" t="s">
-        <v>139</v>
       </c>
       <c r="V14" s="1" t="s">
         <v>139</v>
@@ -2609,8 +2712,14 @@
       <c r="W14" s="1" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="X14" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="Y14" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>149</v>
       </c>
@@ -2642,13 +2751,19 @@
         <f t="shared" si="0"/>
         <v>c(0.01,3.25)</v>
       </c>
-      <c r="T15" s="1" t="s">
+      <c r="S15" s="1">
+        <v>0.01</v>
+      </c>
+      <c r="T15" s="1">
+        <v>0.01</v>
+      </c>
+      <c r="V15" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="V15" s="1" t="s">
+      <c r="X15" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="W15" s="1" t="s">
+      <c r="Y15" s="1" t="s">
         <v>53</v>
       </c>
     </row>
@@ -2662,21 +2777,21 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D24D9501-1928-C24A-A5F8-EF63F20DDAEF}">
   <dimension ref="A1:D34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.33203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="42.1640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.5" style="5" customWidth="1"/>
-    <col min="4" max="4" width="84.6640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="11.33203125" style="5"/>
+    <col min="1" max="1" width="33.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="42.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" style="5" customWidth="1"/>
+    <col min="4" max="4" width="84.7109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="11.28515625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>55</v>
       </c>
@@ -2684,7 +2799,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>57</v>
       </c>
@@ -2692,7 +2807,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>59</v>
       </c>
@@ -2706,7 +2821,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>61</v>
       </c>
@@ -2714,7 +2829,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>62</v>
       </c>
@@ -2722,7 +2837,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>64</v>
       </c>
@@ -2736,7 +2851,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>65</v>
       </c>
@@ -2744,7 +2859,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>67</v>
       </c>
@@ -2752,7 +2867,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>68</v>
       </c>
@@ -2766,7 +2881,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>69</v>
       </c>
@@ -2774,7 +2889,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>70</v>
       </c>
@@ -2782,7 +2897,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>71</v>
       </c>
@@ -2796,7 +2911,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>72</v>
       </c>
@@ -2804,7 +2919,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>73</v>
       </c>
@@ -2812,7 +2927,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>74</v>
       </c>
@@ -2826,7 +2941,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>75</v>
       </c>
@@ -2834,7 +2949,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>76</v>
       </c>
@@ -2842,7 +2957,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>77</v>
       </c>
@@ -2856,7 +2971,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>78</v>
       </c>
@@ -2864,7 +2979,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>80</v>
       </c>
@@ -2872,7 +2987,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
         <v>82</v>
       </c>
@@ -2886,7 +3001,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
         <v>84</v>
       </c>
@@ -2894,7 +3009,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
         <v>85</v>
       </c>
@@ -2902,7 +3017,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
         <v>86</v>
       </c>
@@ -2916,7 +3031,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
         <v>96</v>
       </c>
@@ -2924,7 +3039,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
         <v>97</v>
       </c>
@@ -2932,7 +3047,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
         <v>98</v>
       </c>
@@ -2943,32 +3058,32 @@
         <v>155</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
         <v>92</v>
       </c>

</xml_diff>

<commit_message>
added block randomized clusters to app
</commit_message>
<xml_diff>
--- a/support materials/menuManager.xlsx
+++ b/support materials/menuManager.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10711"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hedbe\Dropbox\Papers\Paper.QEDs\Apps\plannerApp\support materials\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hedbergec/Dropbox/Papers/Paper.QEDs/Apps/plannerApp/support materials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD618F96-4680-4A44-8044-8EA83821097A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC5707BF-004A-6F46-86F3-121ADDAB8796}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31350" yWindow="1515" windowWidth="21600" windowHeight="11145" tabRatio="716" activeTab="6" xr2:uid="{8D89E9AD-B3C8-4CE6-A909-5B9DBA95DCBB}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16260" tabRatio="716" activeTab="6" xr2:uid="{8D89E9AD-B3C8-4CE6-A909-5B9DBA95DCBB}"/>
   </bookViews>
   <sheets>
     <sheet name="readme" sheetId="11" r:id="rId1"/>
@@ -55,7 +55,7 @@
     <author>tc={CA4BCEC2-9B3E-4FC5-B2C2-41BB34B83579}</author>
   </authors>
   <commentList>
-    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{0713FE03-72D3-4E97-9C1A-4F35BCE26CD6}">
+    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{0713FE03-72D3-4E97-9C1A-4F35BCE26CD6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -63,7 +63,7 @@
     which desings use which inputs?</t>
       </text>
     </comment>
-    <comment ref="I1" authorId="1" shapeId="0" xr:uid="{C16FA29C-DF1E-443B-B6F4-2B0EAF1F7A79}">
+    <comment ref="J1" authorId="1" shapeId="0" xr:uid="{C16FA29C-DF1E-443B-B6F4-2B0EAF1F7A79}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -71,7 +71,7 @@
     which inference sets use which inputs?</t>
       </text>
     </comment>
-    <comment ref="J1" authorId="2" shapeId="0" xr:uid="{56996333-72A8-4807-9F7B-A26D365E50ED}">
+    <comment ref="K1" authorId="2" shapeId="0" xr:uid="{56996333-72A8-4807-9F7B-A26D365E50ED}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -79,7 +79,7 @@
     used in no-covariate models?</t>
       </text>
     </comment>
-    <comment ref="K1" authorId="3" shapeId="0" xr:uid="{1242266B-8183-4A71-810B-FA35C112B92A}">
+    <comment ref="L1" authorId="3" shapeId="0" xr:uid="{1242266B-8183-4A71-810B-FA35C112B92A}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -87,7 +87,7 @@
     used in covariate models</t>
       </text>
     </comment>
-    <comment ref="L1" authorId="4" shapeId="0" xr:uid="{AC5243D4-8E3B-4184-AF1F-518836A7A975}">
+    <comment ref="M1" authorId="4" shapeId="0" xr:uid="{AC5243D4-8E3B-4184-AF1F-518836A7A975}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -95,7 +95,7 @@
     used to compute total sample size?</t>
       </text>
     </comment>
-    <comment ref="M1" authorId="5" shapeId="0" xr:uid="{721899ED-7FCC-4F2B-BB22-844D27DA8843}">
+    <comment ref="N1" authorId="5" shapeId="0" xr:uid="{721899ED-7FCC-4F2B-BB22-844D27DA8843}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -103,7 +103,7 @@
     used to compute df?</t>
       </text>
     </comment>
-    <comment ref="N1" authorId="6" shapeId="0" xr:uid="{53AAC73E-37CD-4F93-952F-58532973ACC7}">
+    <comment ref="O1" authorId="6" shapeId="0" xr:uid="{53AAC73E-37CD-4F93-952F-58532973ACC7}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -111,7 +111,7 @@
     Used in Variance Factor?</t>
       </text>
     </comment>
-    <comment ref="Q1" authorId="7" shapeId="0" xr:uid="{404E6D2E-D072-435D-810D-184FE609405B}">
+    <comment ref="R1" authorId="7" shapeId="0" xr:uid="{404E6D2E-D072-435D-810D-184FE609405B}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -119,7 +119,7 @@
     Default Value</t>
       </text>
     </comment>
-    <comment ref="R1" authorId="8" shapeId="0" xr:uid="{1DE218DE-31C8-4B3E-95DD-574166043541}">
+    <comment ref="S1" authorId="8" shapeId="0" xr:uid="{1DE218DE-31C8-4B3E-95DD-574166043541}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -127,7 +127,7 @@
     Not used yet, but made with excel formula</t>
       </text>
     </comment>
-    <comment ref="T1" authorId="9" shapeId="0" xr:uid="{CA4BCEC2-9B3E-4FC5-B2C2-41BB34B83579}">
+    <comment ref="U1" authorId="9" shapeId="0" xr:uid="{CA4BCEC2-9B3E-4FC5-B2C2-41BB34B83579}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -143,6 +143,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={1275E356-8889-4DE3-A9F1-EFFEAADE9EBC}</author>
+    <author>tc={EEF03417-7147-F648-A51C-4C2D4C4E7DB2}</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0" xr:uid="{1275E356-8889-4DE3-A9F1-EFFEAADE9EBC}">
@@ -153,12 +154,20 @@
     the string below are the names for the *.R files created</t>
       </text>
     </comment>
+    <comment ref="B1" authorId="1" shapeId="0" xr:uid="{EEF03417-7147-F648-A51C-4C2D4C4E7DB2}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    place for comments</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="188">
   <si>
     <t>sample</t>
   </si>
@@ -656,13 +665,79 @@
   </si>
   <si>
     <t>ui_step_exact</t>
+  </si>
+  <si>
+    <t>blockedclustered</t>
+  </si>
+  <si>
+    <t>Blocked Randomized with Cluster Assignment</t>
+  </si>
+  <si>
+    <t>k</t>
+  </si>
+  <si>
+    <t>label_blockedclustered</t>
+  </si>
+  <si>
+    <t>Number of intervention group clusters per block</t>
+  </si>
+  <si>
+    <t>Number of comparison  group clusters per block</t>
+  </si>
+  <si>
+    <t>Number individuals per cluster per block</t>
+  </si>
+  <si>
+    <t>Intraclass correlation (ICC) within blocks</t>
+  </si>
+  <si>
+    <t>Variance reduction in outcome (clusters within blocks)</t>
+  </si>
+  <si>
+    <t>blockedclustered_fixed_nocovariate_N</t>
+  </si>
+  <si>
+    <t>blockedclustered_fixed_nocovariate_df</t>
+  </si>
+  <si>
+    <t>blockedclustered_fixed_nocovariate_V</t>
+  </si>
+  <si>
+    <t>blockedclustered_fixed_covariate_N</t>
+  </si>
+  <si>
+    <t>blockedclustered_fixed_covariate_df</t>
+  </si>
+  <si>
+    <t>blockedclustered_fixed_covariate_V</t>
+  </si>
+  <si>
+    <t>df &lt;- k-1</t>
+  </si>
+  <si>
+    <t>N &lt;- k*(mt+mc)*n</t>
+  </si>
+  <si>
+    <t>V &lt;- k*m*n*p*(1-p)*(1/(1+(n-1)*icc))</t>
+  </si>
+  <si>
+    <t>df &lt;- k-1-q</t>
+  </si>
+  <si>
+    <t>V &lt;- k*m*n*p*(1-p)*(1/(1+(n-1)*icc-(R2_1+(n*R2_2-R2_1)*icc)))</t>
+  </si>
+  <si>
+    <t>#expression 30 in Hedges and Rhoads</t>
+  </si>
+  <si>
+    <t>#</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -695,12 +770,6 @@
       <sz val="11"/>
       <name val="Consolas"/>
       <family val="3"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -740,7 +809,7 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="12">
     <dxf>
       <font>
         <b val="0"/>
@@ -898,6 +967,42 @@
         <vertAlign val="baseline"/>
         <sz val="11"/>
         <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
         <name val="Consolas"/>
         <family val="3"/>
         <scheme val="none"/>
@@ -941,9 +1046,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6152DF64-9A11-42D3-B695-178EF7A61CD5}" name="Table3" displayName="Table3" ref="A1:D34" headerRowCount="0" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{14FCBBA3-4721-4280-B533-C0FC542668AA}" name="Column1" headerRowDxfId="7" dataDxfId="6"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6152DF64-9A11-42D3-B695-178EF7A61CD5}" name="Table3" displayName="Table3" ref="A1:E40" headerRowCount="0" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{14FCBBA3-4721-4280-B533-C0FC542668AA}" name="Column1" headerRowDxfId="9" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{325E2793-747D-D245-82E5-0CFCB3777237}" name="Column5" headerRowDxfId="7" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{E90FB251-9DD0-40B0-A06B-487DE170DB7D}" name="Column2" headerRowDxfId="5" dataDxfId="4"/>
     <tableColumn id="3" xr3:uid="{1DDFB4AE-3D35-415F-AC9F-F95F752C46CF}" name="Column3" headerRowDxfId="3" dataDxfId="2"/>
     <tableColumn id="4" xr3:uid="{5BDFB90D-F447-456A-9633-044179DB9760}" name="Column4" headerRowDxfId="1" dataDxfId="0"/>
@@ -1249,34 +1355,34 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="G1" dT="2021-07-10T01:04:10.84" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{0713FE03-72D3-4E97-9C1A-4F35BCE26CD6}">
+  <threadedComment ref="H1" dT="2021-07-10T01:04:10.84" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{0713FE03-72D3-4E97-9C1A-4F35BCE26CD6}">
     <text>which desings use which inputs?</text>
   </threadedComment>
-  <threadedComment ref="I1" dT="2021-07-10T01:04:37.05" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{C16FA29C-DF1E-443B-B6F4-2B0EAF1F7A79}">
+  <threadedComment ref="J1" dT="2021-07-10T01:04:37.05" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{C16FA29C-DF1E-443B-B6F4-2B0EAF1F7A79}">
     <text>which inference sets use which inputs?</text>
   </threadedComment>
-  <threadedComment ref="J1" dT="2021-07-10T00:55:47.10" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{56996333-72A8-4807-9F7B-A26D365E50ED}">
+  <threadedComment ref="K1" dT="2021-07-10T00:55:47.10" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{56996333-72A8-4807-9F7B-A26D365E50ED}">
     <text>used in no-covariate models?</text>
   </threadedComment>
-  <threadedComment ref="K1" dT="2021-07-10T00:55:19.43" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{1242266B-8183-4A71-810B-FA35C112B92A}">
+  <threadedComment ref="L1" dT="2021-07-10T00:55:19.43" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{1242266B-8183-4A71-810B-FA35C112B92A}">
     <text>used in covariate models</text>
   </threadedComment>
-  <threadedComment ref="L1" dT="2021-07-10T00:55:08.33" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{AC5243D4-8E3B-4184-AF1F-518836A7A975}">
+  <threadedComment ref="M1" dT="2021-07-10T00:55:08.33" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{AC5243D4-8E3B-4184-AF1F-518836A7A975}">
     <text>used to compute total sample size?</text>
   </threadedComment>
-  <threadedComment ref="M1" dT="2021-07-10T00:54:10.24" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{721899ED-7FCC-4F2B-BB22-844D27DA8843}">
+  <threadedComment ref="N1" dT="2021-07-10T00:54:10.24" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{721899ED-7FCC-4F2B-BB22-844D27DA8843}">
     <text>used to compute df?</text>
   </threadedComment>
-  <threadedComment ref="N1" dT="2021-07-10T00:53:59.73" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{53AAC73E-37CD-4F93-952F-58532973ACC7}">
+  <threadedComment ref="O1" dT="2021-07-10T00:53:59.73" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{53AAC73E-37CD-4F93-952F-58532973ACC7}">
     <text>Used in Variance Factor?</text>
   </threadedComment>
-  <threadedComment ref="Q1" dT="2021-07-10T00:53:45.02" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{404E6D2E-D072-435D-810D-184FE609405B}">
+  <threadedComment ref="R1" dT="2021-07-10T00:53:45.02" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{404E6D2E-D072-435D-810D-184FE609405B}">
     <text>Default Value</text>
   </threadedComment>
-  <threadedComment ref="R1" dT="2021-07-10T00:53:30.43" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{1DE218DE-31C8-4B3E-95DD-574166043541}">
+  <threadedComment ref="S1" dT="2021-07-10T00:53:30.43" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{1DE218DE-31C8-4B3E-95DD-574166043541}">
     <text>Not used yet, but made with excel formula</text>
   </threadedComment>
-  <threadedComment ref="T1" dT="2021-07-10T00:53:30.43" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{CA4BCEC2-9B3E-4FC5-B2C2-41BB34B83579}">
+  <threadedComment ref="U1" dT="2021-07-10T00:53:30.43" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{CA4BCEC2-9B3E-4FC5-B2C2-41BB34B83579}">
     <text>Not used yet, but made with excel formula</text>
   </threadedComment>
 </ThreadedComments>
@@ -1287,28 +1393,31 @@
   <threadedComment ref="A1" dT="2021-07-10T01:03:40.46" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{1275E356-8889-4DE3-A9F1-EFFEAADE9EBC}">
     <text>the string below are the names for the *.R files created</text>
   </threadedComment>
+  <threadedComment ref="B1" dT="2021-07-15T23:22:05.25" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{EEF03417-7147-F648-A51C-4C2D4C4E7DB2}">
+    <text>place for comments</text>
+  </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C51C3392-495A-4716-B7D0-8CB1570246E2}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.7109375" customWidth="1"/>
+    <col min="1" max="1" width="21.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="str">
         <f>HYPERLINK(sample!A1)</f>
         <v>sample</v>
@@ -1317,7 +1426,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="str">
         <f>HYPERLINK(design!A1)</f>
         <v>design</v>
@@ -1326,7 +1435,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="str">
         <f>HYPERLINK(inference!A1)</f>
         <v>inference</v>
@@ -1335,7 +1444,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="str">
         <f>HYPERLINK(model!A1)</f>
         <v>model</v>
@@ -1344,7 +1453,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="str">
         <f>HYPERLINK(stat!A1)</f>
         <v>stat</v>
@@ -1353,7 +1462,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="str">
         <f>HYPERLINK(input!A1)</f>
         <v>input</v>
@@ -1362,13 +1471,13 @@
         <v>110</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="2"/>
       <c r="C9" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="str">
         <f>HYPERLINK(code!A1,"code")</f>
         <v>code</v>
@@ -1377,7 +1486,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="C11" t="s">
         <v>108</v>
       </c>
@@ -1390,9 +1499,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A96E0447-8401-42C5-BE02-401F505AE938}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1400,7 +1509,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1408,7 +1517,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1423,13 +1532,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62AA0D0E-E4D1-469A-AF1F-085E17D5518F}">
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="29.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -1443,7 +1552,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1454,7 +1563,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1465,7 +1574,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1476,36 +1585,47 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>166</v>
+      </c>
+      <c r="B5" t="s">
+        <v>167</v>
+      </c>
+      <c r="C5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>10</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B6" t="s">
         <v>145</v>
-      </c>
-      <c r="D5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" t="s">
-        <v>146</v>
       </c>
       <c r="D6" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s">
+        <v>146</v>
+      </c>
+      <c r="D7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>93</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B8" t="s">
         <v>147</v>
       </c>
-      <c r="D7" t="b">
+      <c r="D8" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1516,14 +1636,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33C6AD60-7AB8-4CAF-9726-0F1707E818DE}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.140625" customWidth="1"/>
+    <col min="3" max="3" width="5.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -1540,16 +1660,19 @@
         <v>9</v>
       </c>
       <c r="F1" t="s">
+        <v>166</v>
+      </c>
+      <c r="G1" t="s">
         <v>10</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>11</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -1571,8 +1694,11 @@
       <c r="H2" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1593,15 +1719,15 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F39838A5-C062-40CB-BD39-4466E5E1974A}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -1618,16 +1744,19 @@
         <v>9</v>
       </c>
       <c r="F1" t="s">
+        <v>166</v>
+      </c>
+      <c r="G1" t="s">
         <v>10</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>11</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -1652,8 +1781,11 @@
       <c r="H2" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -1667,6 +1799,9 @@
         <v>1</v>
       </c>
       <c r="E3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1677,14 +1812,14 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9306200-6D5D-404E-9AA4-2D83AC7E89FD}">
-  <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>20</v>
       </c>
@@ -1701,16 +1836,19 @@
         <v>9</v>
       </c>
       <c r="F1" t="s">
+        <v>166</v>
+      </c>
+      <c r="G1" t="s">
         <v>10</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>11</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -1735,8 +1873,11 @@
       <c r="H2" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -1761,8 +1902,11 @@
       <c r="H3" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -1785,6 +1929,9 @@
         <v>1</v>
       </c>
       <c r="H4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1796,29 +1943,30 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7085B87C-0BDF-4509-A80F-252767BE3B26}">
-  <dimension ref="A1:Z15"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AB16"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" style="1" customWidth="1"/>
     <col min="3" max="3" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="5.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.28515625" style="1" customWidth="1"/>
-    <col min="8" max="9" width="7.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="7.85546875" style="1" customWidth="1"/>
-    <col min="15" max="16" width="9.140625" style="1" customWidth="1"/>
-    <col min="17" max="17" width="14.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="14.7109375" style="1" customWidth="1"/>
-    <col min="21" max="23" width="49.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="55.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="16384" width="9.140625" style="1"/>
+    <col min="4" max="4" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="5.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.33203125" style="1" customWidth="1"/>
+    <col min="9" max="10" width="7.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="15" width="7.83203125" style="1" customWidth="1"/>
+    <col min="16" max="17" width="9.1640625" style="1" customWidth="1"/>
+    <col min="18" max="18" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="14.6640625" style="1" customWidth="1"/>
+    <col min="22" max="24" width="49.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="49.33203125" style="1" customWidth="1"/>
+    <col min="26" max="27" width="55.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="16384" width="9.1640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>27</v>
       </c>
@@ -1832,938 +1980,1034 @@
         <v>9</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="Z1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="E2" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="K2" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L2" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="M2" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="N2" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="O2" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="P2" s="1">
+        <v>2</v>
+      </c>
+      <c r="Q2" s="1">
+        <v>40</v>
+      </c>
+      <c r="R2" s="1">
+        <v>3</v>
+      </c>
+      <c r="S2" s="1" t="str">
+        <f>_xlfn.CONCAT("c(",P2,",",Q2,")")</f>
+        <v>c(2,40)</v>
+      </c>
+      <c r="T2" s="1">
+        <v>1</v>
+      </c>
+      <c r="U2" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="E2" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H2" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="I2" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="J2" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="K2" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="L2" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="M2" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="N2" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O2" s="1">
+      <c r="C3" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I3" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J3" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="K3" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L3" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="M3" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="N3" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="O3" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="P3" s="1">
         <v>4</v>
       </c>
-      <c r="P2" s="1">
+      <c r="Q3" s="1">
         <v>40</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="R3" s="1">
         <v>10</v>
       </c>
-      <c r="R2" s="1" t="str">
-        <f>_xlfn.CONCAT("c(",O2,",",P2,")")</f>
+      <c r="S3" s="1" t="str">
+        <f>_xlfn.CONCAT("c(",P3,",",Q3,")")</f>
         <v>c(4,40)</v>
       </c>
-      <c r="S2" s="1">
-        <v>1</v>
-      </c>
-      <c r="T2" s="1">
-        <v>1</v>
-      </c>
-      <c r="V2" s="1" t="s">
+      <c r="T3" s="1">
+        <v>1</v>
+      </c>
+      <c r="U3" s="1">
+        <v>1</v>
+      </c>
+      <c r="W3" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="W2" s="1" t="s">
+      <c r="X3" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="X2" s="1" t="s">
+      <c r="Z3" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="Y2" s="1" t="s">
+      <c r="AA3" s="1" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D3" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="F3" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H3" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="I3" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="J3" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="K3" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="L3" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="M3" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="N3" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O3" s="1">
+      <c r="D4" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="E4" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J4" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="K4" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L4" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="M4" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="N4" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="O4" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="P4" s="1">
         <v>2</v>
       </c>
-      <c r="P3" s="1">
+      <c r="Q4" s="1">
         <v>40</v>
       </c>
-      <c r="Q3" s="1">
-        <v>5</v>
-      </c>
-      <c r="R3" s="1" t="str">
-        <f t="shared" ref="R3:R15" si="0">_xlfn.CONCAT("c(",O3,",",P3,")")</f>
+      <c r="R4" s="1">
+        <v>3</v>
+      </c>
+      <c r="S4" s="1" t="str">
+        <f t="shared" ref="S4:S16" si="0">_xlfn.CONCAT("c(",P4,",",Q4,")")</f>
         <v>c(2,40)</v>
       </c>
-      <c r="S3" s="1">
-        <v>1</v>
-      </c>
-      <c r="T3" s="1">
-        <v>1</v>
-      </c>
-      <c r="V3" s="1" t="s">
+      <c r="T4" s="1">
+        <v>1</v>
+      </c>
+      <c r="U4" s="1">
+        <v>1</v>
+      </c>
+      <c r="W4" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="W3" s="1" t="s">
+      <c r="X4" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="X3" s="1" t="s">
+      <c r="Y4" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="Z4" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="Y3" s="1" t="s">
+      <c r="AA4" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D4" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="F4" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H4" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="J4" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="K4" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="L4" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="M4" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="N4" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O4" s="1">
+      <c r="D5" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="E5" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J5" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="K5" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L5" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="M5" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="N5" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="O5" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="P5" s="1">
         <v>2</v>
       </c>
-      <c r="P4" s="1">
+      <c r="Q5" s="1">
         <v>40</v>
       </c>
-      <c r="Q4" s="1">
-        <v>5</v>
-      </c>
-      <c r="R4" s="1" t="str">
+      <c r="R5" s="1">
+        <v>3</v>
+      </c>
+      <c r="S5" s="1" t="str">
         <f t="shared" si="0"/>
         <v>c(2,40)</v>
       </c>
-      <c r="S4" s="1">
-        <v>1</v>
-      </c>
-      <c r="T4" s="1">
-        <v>1</v>
-      </c>
-      <c r="V4" s="1" t="s">
+      <c r="T5" s="1">
+        <v>1</v>
+      </c>
+      <c r="U5" s="1">
+        <v>1</v>
+      </c>
+      <c r="W5" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="W4" s="1" t="s">
+      <c r="X5" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="X4" s="1" t="s">
+      <c r="Y5" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="Z5" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="Y4" s="1" t="s">
+      <c r="AA5" s="1" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D5" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H5" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="J5" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="K5" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="L5" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="M5" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="N5" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O5" s="1">
+      <c r="D6" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="E6" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I6" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J6" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="K6" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L6" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="M6" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="N6" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="O6" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="P6" s="1">
         <v>4</v>
       </c>
-      <c r="P5" s="1">
+      <c r="Q6" s="1">
         <v>150</v>
       </c>
-      <c r="Q5" s="1">
-        <v>40</v>
-      </c>
-      <c r="R5" s="1" t="str">
+      <c r="R6" s="1">
+        <v>30</v>
+      </c>
+      <c r="S6" s="1" t="str">
         <f t="shared" si="0"/>
         <v>c(4,150)</v>
       </c>
-      <c r="S5" s="1">
-        <v>1</v>
-      </c>
-      <c r="T5" s="1">
-        <v>1</v>
-      </c>
-      <c r="V5" s="1" t="s">
+      <c r="T6" s="1">
+        <v>1</v>
+      </c>
+      <c r="U6" s="1">
+        <v>1</v>
+      </c>
+      <c r="W6" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="W5" s="1" t="s">
+      <c r="X6" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="X5" s="1" t="s">
+      <c r="Y6" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="Z6" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="Y5" s="1" t="s">
+      <c r="AA6" s="1" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C6" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="G6" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H6" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="I6" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="J6" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="K6" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="L6" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="M6" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="N6" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O6" s="1">
+      <c r="B7" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="C7" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I7" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J7" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="K7" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L7" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="M7" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="N7" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="O7" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="P7" s="1">
         <v>2</v>
       </c>
-      <c r="P6" s="1">
+      <c r="Q7" s="1">
         <v>150</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="R7" s="1">
         <v>20</v>
       </c>
-      <c r="R6" s="1" t="str">
+      <c r="S7" s="1" t="str">
         <f t="shared" si="0"/>
         <v>c(2,150)</v>
       </c>
-      <c r="S6" s="1">
-        <v>1</v>
-      </c>
-      <c r="T6" s="1">
-        <v>1</v>
-      </c>
-      <c r="U6" s="1" t="s">
+      <c r="T7" s="1">
+        <v>1</v>
+      </c>
+      <c r="U7" s="1">
+        <v>1</v>
+      </c>
+      <c r="V7" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="V6" s="1" t="s">
+      <c r="W7" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="W6" s="1" t="s">
+      <c r="X7" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="X6" s="1" t="s">
+      <c r="Z7" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="Y6" s="1" t="s">
+      <c r="AA7" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="Z6" s="1" t="s">
+      <c r="AB7" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B7" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C7" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="G7" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H7" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="I7" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="J7" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="K7" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="L7" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="M7" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="N7" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O7" s="1">
+      <c r="B8" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="C8" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I8" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J8" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="K8" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L8" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="M8" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="N8" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="O8" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="P8" s="1">
         <v>2</v>
       </c>
-      <c r="P7" s="1">
+      <c r="Q8" s="1">
         <v>150</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="R8" s="1">
         <v>20</v>
       </c>
-      <c r="R7" s="1" t="str">
+      <c r="S8" s="1" t="str">
         <f t="shared" si="0"/>
         <v>c(2,150)</v>
       </c>
-      <c r="S7" s="1">
-        <v>1</v>
-      </c>
-      <c r="T7" s="1">
-        <v>1</v>
-      </c>
-      <c r="U7" s="1" t="s">
+      <c r="T8" s="1">
+        <v>1</v>
+      </c>
+      <c r="U8" s="1">
+        <v>1</v>
+      </c>
+      <c r="V8" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="V7" s="1" t="s">
+      <c r="W8" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="W7" s="1" t="s">
+      <c r="X8" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="X7" s="1" t="s">
+      <c r="Z8" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="Y7" s="1" t="s">
+      <c r="AA8" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="Z7" s="1" t="s">
+      <c r="AB8" s="1" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E8" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="F8" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H8" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="I8" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="J8" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="K8" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="L8" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="M8" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="N8" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O8" s="1">
+      <c r="F9" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I9" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J9" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="K9" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L9" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="M9" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="N9" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="O9" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="P9" s="1">
         <v>2</v>
       </c>
-      <c r="P8" s="1">
+      <c r="Q9" s="1">
         <v>100</v>
       </c>
-      <c r="Q8" s="1">
-        <f>O8+2</f>
+      <c r="R9" s="1">
+        <f>P9+2</f>
         <v>4</v>
       </c>
-      <c r="R8" s="1" t="str">
+      <c r="S9" s="1" t="str">
         <f t="shared" si="0"/>
         <v>c(2,100)</v>
       </c>
-      <c r="S8" s="1">
-        <v>1</v>
-      </c>
-      <c r="T8" s="1">
-        <v>1</v>
-      </c>
-      <c r="V8" s="1" t="s">
+      <c r="T9" s="1">
+        <v>1</v>
+      </c>
+      <c r="U9" s="1">
+        <v>1</v>
+      </c>
+      <c r="W9" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="W8" s="1" t="s">
+      <c r="X9" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="X8" s="1" t="s">
+      <c r="Z9" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="Y8" s="1" t="s">
+      <c r="AA9" s="1" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="E9" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="F9" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H9" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="I9" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="J9" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="K9" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="L9" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="M9" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="N9" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O9" s="1">
+      <c r="F10" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="G10" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I10" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J10" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="K10" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L10" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="M10" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="N10" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="O10" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="P10" s="1">
         <v>2</v>
       </c>
-      <c r="P9" s="1">
+      <c r="Q10" s="1">
         <v>100</v>
       </c>
-      <c r="Q9" s="1">
-        <f>O9+2</f>
+      <c r="R10" s="1">
+        <f>P10+2</f>
         <v>4</v>
       </c>
-      <c r="R9" s="1" t="str">
+      <c r="S10" s="1" t="str">
         <f t="shared" si="0"/>
         <v>c(2,100)</v>
       </c>
-      <c r="S9" s="1">
-        <v>1</v>
-      </c>
-      <c r="T9" s="1">
-        <v>1</v>
-      </c>
-      <c r="V9" s="1" t="s">
+      <c r="T10" s="1">
+        <v>1</v>
+      </c>
+      <c r="U10" s="1">
+        <v>1</v>
+      </c>
+      <c r="W10" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="W9" s="1" t="s">
+      <c r="X10" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="X9" s="1" t="s">
+      <c r="Z10" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="Y9" s="1" t="s">
+      <c r="AA10" s="1" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C10" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="D10" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="E10" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="F10" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H10" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="I10" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="J10" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="K10" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="N10" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O10" s="1">
+      <c r="C11" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D11" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="E11" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F11" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="G11" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I11" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J11" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="K11" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L11" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="O11" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="P11" s="1">
         <v>0.01</v>
       </c>
-      <c r="P10" s="1">
+      <c r="Q11" s="1">
         <v>0.2</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="R11" s="1">
         <v>0.1</v>
       </c>
-      <c r="R10" s="1" t="str">
+      <c r="S11" s="1" t="str">
         <f t="shared" si="0"/>
         <v>c(0.01,0.2)</v>
       </c>
-      <c r="S10" s="1">
+      <c r="T11" s="1">
         <v>0.01</v>
       </c>
-      <c r="T10" s="1">
+      <c r="U11" s="1">
         <v>0.01</v>
       </c>
-      <c r="V10" s="1" t="s">
+      <c r="W11" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="W10" s="1" t="s">
+      <c r="X11" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="X10" s="1" t="s">
+      <c r="Y11" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="Z11" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="Y10" s="1" t="s">
+      <c r="AA11" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B11" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C11" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="D11" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H11" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="I11" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="K11" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="N11" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O11" s="1">
+      <c r="B12" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="C12" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D12" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="E12" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I12" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J12" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L12" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="O12" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="P12" s="1">
         <v>0</v>
       </c>
-      <c r="P11" s="1">
+      <c r="Q12" s="1">
         <v>0.99</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="R12" s="1">
         <v>0.2</v>
       </c>
-      <c r="R11" s="1" t="str">
+      <c r="S12" s="1" t="str">
         <f t="shared" si="0"/>
         <v>c(0,0.99)</v>
       </c>
-      <c r="S11" s="1">
+      <c r="T12" s="1">
         <v>0.01</v>
       </c>
-      <c r="T11" s="1">
+      <c r="U12" s="1">
         <v>0.01</v>
       </c>
-      <c r="U11" s="1" t="s">
+      <c r="V12" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="V11" s="1" t="s">
+      <c r="W12" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="W11" s="1" t="s">
+      <c r="X12" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="X11" s="1" t="s">
+      <c r="Y12" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="Y11" s="1" t="s">
+      <c r="Z12" s="1" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="AA12" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C12" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="D12" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="I12" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="K12" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="N12" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O12" s="1">
+      <c r="C13" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D13" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="E13" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J13" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L13" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="O13" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="P13" s="1">
         <v>0</v>
       </c>
-      <c r="P12" s="1">
+      <c r="Q13" s="1">
         <v>0.99</v>
       </c>
-      <c r="Q12" s="1">
+      <c r="R13" s="1">
         <v>0.2</v>
       </c>
-      <c r="R12" s="1" t="str">
+      <c r="S13" s="1" t="str">
         <f t="shared" si="0"/>
         <v>c(0,0.99)</v>
       </c>
-      <c r="S12" s="1">
+      <c r="T13" s="1">
         <v>0.01</v>
       </c>
-      <c r="T12" s="1">
+      <c r="U13" s="1">
         <v>0.01</v>
       </c>
-      <c r="V12" s="1" t="s">
+      <c r="W13" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="W12" s="1" t="s">
+      <c r="X13" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="X12" s="3" t="s">
+      <c r="Y13" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="Z13" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="Y12" s="3" t="s">
+      <c r="AA13" s="3" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="E13" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="F13" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="G13" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H13" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="I13" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="J13" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="K13" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="N13" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O13" s="1">
+      <c r="F14" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="G14" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="H14" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I14" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J14" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="K14" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L14" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="O14" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="P14" s="1">
         <v>0</v>
       </c>
-      <c r="P13" s="1">
+      <c r="Q14" s="1">
         <v>0.99</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="R14" s="1">
         <v>0.25</v>
       </c>
-      <c r="R13" s="1" t="str">
+      <c r="S14" s="1" t="str">
         <f t="shared" si="0"/>
         <v>c(0,0.99)</v>
       </c>
-      <c r="S13" s="1">
+      <c r="T14" s="1">
         <v>0.01</v>
       </c>
-      <c r="T13" s="1">
+      <c r="U14" s="1">
         <v>0.01</v>
       </c>
-      <c r="V13" s="1" t="s">
+      <c r="W14" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="W13" s="1" t="s">
+      <c r="X14" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="X13" s="1" t="s">
+      <c r="Z14" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="Y13" s="1" t="s">
+      <c r="AA14" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="Z13" s="1" t="s">
+      <c r="AB14" s="1" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B14" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C14" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="D14" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H14" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="I14" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="K14" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="M14" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="N14" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O14" s="1">
-        <v>1</v>
-      </c>
-      <c r="P14" s="1">
+      <c r="B15" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="C15" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D15" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="E15" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I15" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J15" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L15" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="N15" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="O15" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="P15" s="1">
+        <v>1</v>
+      </c>
+      <c r="Q15" s="1">
         <v>6</v>
       </c>
-      <c r="Q14" s="1">
-        <v>1</v>
-      </c>
-      <c r="R14" s="1" t="str">
+      <c r="R15" s="1">
+        <v>1</v>
+      </c>
+      <c r="S15" s="1" t="str">
         <f t="shared" si="0"/>
         <v>c(1,6)</v>
       </c>
-      <c r="S14" s="1">
-        <v>1</v>
-      </c>
-      <c r="T14" s="1">
-        <v>1</v>
-      </c>
-      <c r="U14" s="1" t="s">
+      <c r="T15" s="1">
+        <v>1</v>
+      </c>
+      <c r="U15" s="1">
+        <v>1</v>
+      </c>
+      <c r="V15" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="V14" s="1" t="s">
+      <c r="W15" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="W14" s="1" t="s">
+      <c r="X15" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="X14" s="1" t="s">
+      <c r="Y15" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="Y14" s="1" t="s">
+      <c r="Z15" s="1" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+      <c r="AA15" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="C15" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="I15" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="J15" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="K15" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="N15" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O15" s="1">
+      <c r="C16" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J16" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="K16" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L16" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="O16" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="P16" s="1">
         <v>0.01</v>
       </c>
-      <c r="P15" s="1">
+      <c r="Q16" s="1">
         <v>3.25</v>
       </c>
-      <c r="Q15" s="1">
+      <c r="R16" s="1">
         <v>0.15</v>
       </c>
-      <c r="R15" s="1" t="str">
+      <c r="S16" s="1" t="str">
         <f t="shared" si="0"/>
         <v>c(0.01,3.25)</v>
       </c>
-      <c r="S15" s="1">
+      <c r="T16" s="1">
         <v>0.01</v>
       </c>
-      <c r="T15" s="1">
+      <c r="U16" s="1">
         <v>0.01</v>
       </c>
-      <c r="V15" s="1" t="s">
+      <c r="W16" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="X15" s="1" t="s">
+      <c r="Z16" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="Y15" s="1" t="s">
+      <c r="AA16" s="1" t="s">
         <v>53</v>
       </c>
     </row>
@@ -2776,315 +3020,472 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D24D9501-1928-C24A-A5F8-EF63F20DDAEF}">
-  <dimension ref="A1:D34"/>
-  <sheetFormatPr defaultColWidth="11.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E40"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.33203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="33.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="42.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.42578125" style="5" customWidth="1"/>
-    <col min="4" max="4" width="84.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="11.28515625" style="5"/>
+    <col min="1" max="1" width="33.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.5" style="4" customWidth="1"/>
+    <col min="3" max="3" width="42.1640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5" style="5" customWidth="1"/>
+    <col min="5" max="5" width="84.6640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="11.33203125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="D7" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="E7" s="5" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="D10" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="E10" s="5" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="E13" s="5" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C16" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="D16" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="E16" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="D19" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="E19" s="5" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C22" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="D22" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="E22" s="5" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C24" s="5" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C25" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="D25" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="E25" s="5" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B32" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C32" s="5" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="4" t="s">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B33" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C33" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="4" t="s">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="B34" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="C34" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="D28" s="5" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="4" t="s">
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" s="4" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="4" t="s">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" s="4" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" s="4" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="4" t="s">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" s="4" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" s="4" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" s="4" t="s">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" s="4" t="s">
         <v>92</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed blockedclustered df with cov
</commit_message>
<xml_diff>
--- a/support materials/menuManager.xlsx
+++ b/support materials/menuManager.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hedbergec/Dropbox/Papers/Paper.QEDs/Apps/plannerApp/support materials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC5707BF-004A-6F46-86F3-121ADDAB8796}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D05F0C12-F702-A34B-930A-5EB5E0F2644F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16260" tabRatio="716" activeTab="6" xr2:uid="{8D89E9AD-B3C8-4CE6-A909-5B9DBA95DCBB}"/>
   </bookViews>
@@ -2078,7 +2078,7 @@
         <v>1</v>
       </c>
       <c r="P2" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q2" s="1">
         <v>40</v>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="S2" s="1" t="str">
         <f>_xlfn.CONCAT("c(",P2,",",Q2,")")</f>
-        <v>c(2,40)</v>
+        <v>c(3,40)</v>
       </c>
       <c r="T2" s="1">
         <v>1</v>
@@ -2787,6 +2787,9 @@
       <c r="E13" s="1" t="b">
         <v>1</v>
       </c>
+      <c r="I13" s="1" t="b">
+        <v>1</v>
+      </c>
       <c r="J13" s="1" t="b">
         <v>1</v>
       </c>
@@ -2929,14 +2932,14 @@
         <v>1</v>
       </c>
       <c r="Q15" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R15" s="1">
         <v>1</v>
       </c>
       <c r="S15" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>c(1,6)</v>
+        <v>c(1,3)</v>
       </c>
       <c r="T15" s="1">
         <v>1</v>

</xml_diff>

<commit_message>
updates to blocked models, labs
</commit_message>
<xml_diff>
--- a/support materials/menuManager.xlsx
+++ b/support materials/menuManager.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hedbergec/Dropbox/Papers/Paper.QEDs/Apps/plannerApp/support materials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D05F0C12-F702-A34B-930A-5EB5E0F2644F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F85E11FC-CDBE-BE4C-A105-436F75565344}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16260" tabRatio="716" activeTab="6" xr2:uid="{8D89E9AD-B3C8-4CE6-A909-5B9DBA95DCBB}"/>
+    <workbookView xWindow="9560" yWindow="1700" windowWidth="28800" windowHeight="16260" tabRatio="716" activeTab="2" xr2:uid="{8D89E9AD-B3C8-4CE6-A909-5B9DBA95DCBB}"/>
   </bookViews>
   <sheets>
     <sheet name="readme" sheetId="11" r:id="rId1"/>
@@ -55,7 +55,7 @@
     <author>tc={CA4BCEC2-9B3E-4FC5-B2C2-41BB34B83579}</author>
   </authors>
   <commentList>
-    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{0713FE03-72D3-4E97-9C1A-4F35BCE26CD6}">
+    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{0713FE03-72D3-4E97-9C1A-4F35BCE26CD6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -63,7 +63,7 @@
     which desings use which inputs?</t>
       </text>
     </comment>
-    <comment ref="J1" authorId="1" shapeId="0" xr:uid="{C16FA29C-DF1E-443B-B6F4-2B0EAF1F7A79}">
+    <comment ref="K1" authorId="1" shapeId="0" xr:uid="{C16FA29C-DF1E-443B-B6F4-2B0EAF1F7A79}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -71,7 +71,7 @@
     which inference sets use which inputs?</t>
       </text>
     </comment>
-    <comment ref="K1" authorId="2" shapeId="0" xr:uid="{56996333-72A8-4807-9F7B-A26D365E50ED}">
+    <comment ref="L1" authorId="2" shapeId="0" xr:uid="{56996333-72A8-4807-9F7B-A26D365E50ED}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -79,7 +79,7 @@
     used in no-covariate models?</t>
       </text>
     </comment>
-    <comment ref="L1" authorId="3" shapeId="0" xr:uid="{1242266B-8183-4A71-810B-FA35C112B92A}">
+    <comment ref="M1" authorId="3" shapeId="0" xr:uid="{1242266B-8183-4A71-810B-FA35C112B92A}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -87,7 +87,7 @@
     used in covariate models</t>
       </text>
     </comment>
-    <comment ref="M1" authorId="4" shapeId="0" xr:uid="{AC5243D4-8E3B-4184-AF1F-518836A7A975}">
+    <comment ref="N1" authorId="4" shapeId="0" xr:uid="{AC5243D4-8E3B-4184-AF1F-518836A7A975}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -95,7 +95,7 @@
     used to compute total sample size?</t>
       </text>
     </comment>
-    <comment ref="N1" authorId="5" shapeId="0" xr:uid="{721899ED-7FCC-4F2B-BB22-844D27DA8843}">
+    <comment ref="O1" authorId="5" shapeId="0" xr:uid="{721899ED-7FCC-4F2B-BB22-844D27DA8843}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -103,7 +103,7 @@
     used to compute df?</t>
       </text>
     </comment>
-    <comment ref="O1" authorId="6" shapeId="0" xr:uid="{53AAC73E-37CD-4F93-952F-58532973ACC7}">
+    <comment ref="P1" authorId="6" shapeId="0" xr:uid="{53AAC73E-37CD-4F93-952F-58532973ACC7}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -111,7 +111,7 @@
     Used in Variance Factor?</t>
       </text>
     </comment>
-    <comment ref="R1" authorId="7" shapeId="0" xr:uid="{404E6D2E-D072-435D-810D-184FE609405B}">
+    <comment ref="S1" authorId="7" shapeId="0" xr:uid="{404E6D2E-D072-435D-810D-184FE609405B}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -119,7 +119,7 @@
     Default Value</t>
       </text>
     </comment>
-    <comment ref="S1" authorId="8" shapeId="0" xr:uid="{1DE218DE-31C8-4B3E-95DD-574166043541}">
+    <comment ref="T1" authorId="8" shapeId="0" xr:uid="{1DE218DE-31C8-4B3E-95DD-574166043541}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -127,7 +127,7 @@
     Not used yet, but made with excel formula</t>
       </text>
     </comment>
-    <comment ref="U1" authorId="9" shapeId="0" xr:uid="{CA4BCEC2-9B3E-4FC5-B2C2-41BB34B83579}">
+    <comment ref="V1" authorId="9" shapeId="0" xr:uid="{CA4BCEC2-9B3E-4FC5-B2C2-41BB34B83579}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -167,7 +167,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="197">
   <si>
     <t>sample</t>
   </si>
@@ -502,9 +502,6 @@
     <t>&lt;- This sheet notes which designs, inference, model, etc., need which elements for stats</t>
   </si>
   <si>
-    <t>Blocked Random Assignment</t>
-  </si>
-  <si>
     <t>Clustered Random Assignment</t>
   </si>
   <si>
@@ -535,12 +532,6 @@
     <t>Number of blocks</t>
   </si>
   <si>
-    <t>Number of intervention group blocks</t>
-  </si>
-  <si>
-    <t>Number of comparison group blocks</t>
-  </si>
-  <si>
     <t>Intraclass correlation (ICC)</t>
   </si>
   <si>
@@ -559,9 +550,6 @@
     <t>Number individuals per  cluster</t>
   </si>
   <si>
-    <t>Number individuals per  block</t>
-  </si>
-  <si>
     <t>Number of comparison  group individuals per  block</t>
   </si>
   <si>
@@ -670,9 +658,6 @@
     <t>blockedclustered</t>
   </si>
   <si>
-    <t>Blocked Randomized with Cluster Assignment</t>
-  </si>
-  <si>
     <t>k</t>
   </si>
   <si>
@@ -731,6 +716,48 @@
   </si>
   <si>
     <t>#</t>
+  </si>
+  <si>
+    <t>dummyblocked</t>
+  </si>
+  <si>
+    <t>label_dummyblocked</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Variance explained by block effects</t>
+  </si>
+  <si>
+    <t>dummyblocked_fixed_nocovariate_N</t>
+  </si>
+  <si>
+    <t>dummyblocked_fixed_nocovariate_df</t>
+  </si>
+  <si>
+    <t>dummyblocked_fixed_nocovariate_V</t>
+  </si>
+  <si>
+    <t>dummyblocked_fixed_covariate_N</t>
+  </si>
+  <si>
+    <t>dummyblocked_fixed_covariate_df</t>
+  </si>
+  <si>
+    <t>dummyblocked_fixed_covariate_V</t>
+  </si>
+  <si>
+    <t>V &lt;- m*n*p*(1-p)*(1/(1-icc))*(1/(1-R2_1))</t>
+  </si>
+  <si>
+    <t>Blocked Random Assignment with Random Effects</t>
+  </si>
+  <si>
+    <t>Blocked Random Assignment with Fixed Effects</t>
+  </si>
+  <si>
+    <t>Blocked Random Cluster Assignment (fixed block effects and random cluster effects)</t>
   </si>
 </sst>
 </file>
@@ -1046,7 +1073,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6152DF64-9A11-42D3-B695-178EF7A61CD5}" name="Table3" displayName="Table3" ref="A1:E40" headerRowCount="0" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6152DF64-9A11-42D3-B695-178EF7A61CD5}" name="Table3" displayName="Table3" ref="A1:E46" headerRowCount="0" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{14FCBBA3-4721-4280-B533-C0FC542668AA}" name="Column1" headerRowDxfId="9" dataDxfId="8"/>
     <tableColumn id="5" xr3:uid="{325E2793-747D-D245-82E5-0CFCB3777237}" name="Column5" headerRowDxfId="7" dataDxfId="6"/>
@@ -1355,34 +1382,34 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="H1" dT="2021-07-10T01:04:10.84" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{0713FE03-72D3-4E97-9C1A-4F35BCE26CD6}">
+  <threadedComment ref="I1" dT="2021-07-10T01:04:10.84" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{0713FE03-72D3-4E97-9C1A-4F35BCE26CD6}">
     <text>which desings use which inputs?</text>
   </threadedComment>
-  <threadedComment ref="J1" dT="2021-07-10T01:04:37.05" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{C16FA29C-DF1E-443B-B6F4-2B0EAF1F7A79}">
+  <threadedComment ref="K1" dT="2021-07-10T01:04:37.05" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{C16FA29C-DF1E-443B-B6F4-2B0EAF1F7A79}">
     <text>which inference sets use which inputs?</text>
   </threadedComment>
-  <threadedComment ref="K1" dT="2021-07-10T00:55:47.10" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{56996333-72A8-4807-9F7B-A26D365E50ED}">
+  <threadedComment ref="L1" dT="2021-07-10T00:55:47.10" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{56996333-72A8-4807-9F7B-A26D365E50ED}">
     <text>used in no-covariate models?</text>
   </threadedComment>
-  <threadedComment ref="L1" dT="2021-07-10T00:55:19.43" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{1242266B-8183-4A71-810B-FA35C112B92A}">
+  <threadedComment ref="M1" dT="2021-07-10T00:55:19.43" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{1242266B-8183-4A71-810B-FA35C112B92A}">
     <text>used in covariate models</text>
   </threadedComment>
-  <threadedComment ref="M1" dT="2021-07-10T00:55:08.33" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{AC5243D4-8E3B-4184-AF1F-518836A7A975}">
+  <threadedComment ref="N1" dT="2021-07-10T00:55:08.33" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{AC5243D4-8E3B-4184-AF1F-518836A7A975}">
     <text>used to compute total sample size?</text>
   </threadedComment>
-  <threadedComment ref="N1" dT="2021-07-10T00:54:10.24" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{721899ED-7FCC-4F2B-BB22-844D27DA8843}">
+  <threadedComment ref="O1" dT="2021-07-10T00:54:10.24" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{721899ED-7FCC-4F2B-BB22-844D27DA8843}">
     <text>used to compute df?</text>
   </threadedComment>
-  <threadedComment ref="O1" dT="2021-07-10T00:53:59.73" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{53AAC73E-37CD-4F93-952F-58532973ACC7}">
+  <threadedComment ref="P1" dT="2021-07-10T00:53:59.73" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{53AAC73E-37CD-4F93-952F-58532973ACC7}">
     <text>Used in Variance Factor?</text>
   </threadedComment>
-  <threadedComment ref="R1" dT="2021-07-10T00:53:45.02" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{404E6D2E-D072-435D-810D-184FE609405B}">
+  <threadedComment ref="S1" dT="2021-07-10T00:53:45.02" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{404E6D2E-D072-435D-810D-184FE609405B}">
     <text>Default Value</text>
   </threadedComment>
-  <threadedComment ref="S1" dT="2021-07-10T00:53:30.43" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{1DE218DE-31C8-4B3E-95DD-574166043541}">
+  <threadedComment ref="T1" dT="2021-07-10T00:53:30.43" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{1DE218DE-31C8-4B3E-95DD-574166043541}">
     <text>Not used yet, but made with excel formula</text>
   </threadedComment>
-  <threadedComment ref="U1" dT="2021-07-10T00:53:30.43" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{CA4BCEC2-9B3E-4FC5-B2C2-41BB34B83579}">
+  <threadedComment ref="V1" dT="2021-07-10T00:53:30.43" personId="{65A658BA-1FAC-4714-A260-E36CAA09F76D}" id="{CA4BCEC2-9B3E-4FC5-B2C2-41BB34B83579}">
     <text>Not used yet, but made with excel formula</text>
   </threadedComment>
 </ThreadedComments>
@@ -1532,7 +1559,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62AA0D0E-E4D1-469A-AF1F-085E17D5518F}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="29.33203125" bestFit="1" customWidth="1"/>
@@ -1557,7 +1584,7 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
@@ -1565,10 +1592,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>183</v>
       </c>
       <c r="B3" t="s">
-        <v>111</v>
+        <v>195</v>
       </c>
       <c r="C3" t="b">
         <v>1</v>
@@ -1576,10 +1603,10 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>112</v>
+        <v>194</v>
       </c>
       <c r="C4" t="b">
         <v>1</v>
@@ -1587,10 +1614,10 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>166</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>167</v>
+        <v>111</v>
       </c>
       <c r="C5" t="b">
         <v>1</v>
@@ -1598,21 +1625,21 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>162</v>
       </c>
       <c r="B6" t="s">
-        <v>145</v>
-      </c>
-      <c r="D6" t="b">
-        <v>0</v>
+        <v>196</v>
+      </c>
+      <c r="C6" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="D7" t="b">
         <v>0</v>
@@ -1620,12 +1647,23 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" t="s">
+        <v>142</v>
+      </c>
+      <c r="D8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>93</v>
       </c>
-      <c r="B8" t="s">
-        <v>147</v>
-      </c>
-      <c r="D8" t="b">
+      <c r="B9" t="s">
+        <v>143</v>
+      </c>
+      <c r="D9" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1636,14 +1674,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33C6AD60-7AB8-4CAF-9726-0F1707E818DE}">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.1640625" customWidth="1"/>
+    <col min="3" max="4" width="5.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -1657,22 +1695,25 @@
         <v>8</v>
       </c>
       <c r="E1" t="s">
+        <v>183</v>
+      </c>
+      <c r="F1" t="s">
         <v>9</v>
       </c>
-      <c r="F1" t="s">
-        <v>166</v>
-      </c>
       <c r="G1" t="s">
+        <v>162</v>
+      </c>
+      <c r="H1" t="s">
         <v>10</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>11</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -1682,10 +1723,7 @@
       <c r="C2" t="b">
         <v>1</v>
       </c>
-      <c r="D2" t="b">
-        <v>1</v>
-      </c>
-      <c r="F2" t="b">
+      <c r="E2" t="b">
         <v>1</v>
       </c>
       <c r="G2" t="b">
@@ -1697,8 +1735,11 @@
       <c r="I2" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1708,7 +1749,7 @@
       <c r="D3" t="b">
         <v>1</v>
       </c>
-      <c r="E3" t="b">
+      <c r="F3" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1719,7 +1760,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F39838A5-C062-40CB-BD39-4466E5E1974A}">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
@@ -1727,7 +1768,7 @@
     <col min="3" max="3" width="5.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -1741,27 +1782,30 @@
         <v>8</v>
       </c>
       <c r="E1" t="s">
+        <v>183</v>
+      </c>
+      <c r="F1" t="s">
         <v>9</v>
       </c>
-      <c r="F1" t="s">
-        <v>166</v>
-      </c>
       <c r="G1" t="s">
+        <v>162</v>
+      </c>
+      <c r="H1" t="s">
         <v>10</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>11</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
@@ -1784,13 +1828,16 @@
       <c r="I2" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C3" t="b">
         <v>1</v>
@@ -1802,6 +1849,9 @@
         <v>1</v>
       </c>
       <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1812,14 +1862,14 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9306200-6D5D-404E-9AA4-2D83AC7E89FD}">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="22.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>20</v>
       </c>
@@ -1833,22 +1883,25 @@
         <v>8</v>
       </c>
       <c r="E1" t="s">
+        <v>183</v>
+      </c>
+      <c r="F1" t="s">
         <v>9</v>
       </c>
-      <c r="F1" t="s">
-        <v>166</v>
-      </c>
       <c r="G1" t="s">
+        <v>162</v>
+      </c>
+      <c r="H1" t="s">
         <v>10</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>11</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -1876,8 +1929,11 @@
       <c r="I2" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -1905,8 +1961,11 @@
       <c r="I3" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -1932,6 +1991,9 @@
         <v>1</v>
       </c>
       <c r="I4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J4" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1943,30 +2005,32 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7085B87C-0BDF-4509-A80F-252767BE3B26}">
-  <dimension ref="A1:AB16"/>
+  <dimension ref="A1:AD16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" style="1" customWidth="1"/>
-    <col min="3" max="3" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="5.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.33203125" style="1" customWidth="1"/>
-    <col min="9" max="10" width="7.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="15" width="7.83203125" style="1" customWidth="1"/>
-    <col min="16" max="17" width="9.1640625" style="1" customWidth="1"/>
-    <col min="18" max="18" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="21" width="14.6640625" style="1" customWidth="1"/>
-    <col min="22" max="24" width="49.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="8" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="5.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.33203125" style="1" customWidth="1"/>
+    <col min="10" max="11" width="7.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="16" width="7.83203125" style="1" customWidth="1"/>
+    <col min="17" max="18" width="9.1640625" style="1" customWidth="1"/>
+    <col min="19" max="19" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="22" width="14.6640625" style="1" customWidth="1"/>
+    <col min="23" max="24" width="49.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="49.33203125" style="1" customWidth="1"/>
-    <col min="26" max="27" width="55.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="16384" width="9.1640625" style="1"/>
+    <col min="26" max="26" width="49.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="49.33203125" style="1" customWidth="1"/>
+    <col min="28" max="29" width="55.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="30" max="16384" width="9.1640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>27</v>
       </c>
@@ -1977,92 +2041,95 @@
         <v>8</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>166</v>
-      </c>
       <c r="F1" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="T1" s="1" t="s">
-        <v>165</v>
-      </c>
       <c r="U1" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA1" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="V1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="E2" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="I2" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="K2" s="1" t="b">
+        <v>163</v>
+      </c>
+      <c r="F2" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J2" s="1" t="b">
         <v>1</v>
       </c>
       <c r="L2" s="1" t="b">
@@ -2077,40 +2144,43 @@
       <c r="O2" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="1">
         <v>3</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="R2" s="1">
         <v>40</v>
       </c>
-      <c r="R2" s="1">
+      <c r="S2" s="1">
         <v>3</v>
       </c>
-      <c r="S2" s="1" t="str">
-        <f>_xlfn.CONCAT("c(",P2,",",Q2,")")</f>
+      <c r="T2" s="1" t="str">
+        <f>_xlfn.CONCAT("c(",Q2,",",R2,")")</f>
         <v>c(3,40)</v>
       </c>
-      <c r="T2" s="1">
-        <v>1</v>
-      </c>
       <c r="U2" s="1">
         <v>1</v>
       </c>
-      <c r="Y2" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="V2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>37</v>
       </c>
       <c r="C3" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="F3" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="I3" s="1" t="b">
+      <c r="D3" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" s="1" t="b">
         <v>1</v>
       </c>
       <c r="J3" s="1" t="b">
@@ -2131,52 +2201,55 @@
       <c r="O3" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q3" s="1">
         <v>4</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="R3" s="1">
         <v>40</v>
       </c>
-      <c r="R3" s="1">
-        <v>10</v>
-      </c>
-      <c r="S3" s="1" t="str">
-        <f>_xlfn.CONCAT("c(",P3,",",Q3,")")</f>
+      <c r="S3" s="1">
+        <v>5</v>
+      </c>
+      <c r="T3" s="1" t="str">
+        <f>_xlfn.CONCAT("c(",Q3,",",R3,")")</f>
         <v>c(4,40)</v>
       </c>
-      <c r="T3" s="1">
-        <v>1</v>
-      </c>
       <c r="U3" s="1">
         <v>1</v>
       </c>
-      <c r="W3" s="1" t="s">
-        <v>121</v>
+      <c r="V3" s="1">
+        <v>1</v>
       </c>
       <c r="X3" s="1" t="s">
-        <v>126</v>
+        <v>120</v>
+      </c>
+      <c r="Y3" s="1" t="s">
+        <v>120</v>
       </c>
       <c r="Z3" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="AA3" s="1" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.2">
+        <v>123</v>
+      </c>
+      <c r="AB3" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="AC3" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="4" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D4" s="1" t="b">
-        <v>1</v>
-      </c>
       <c r="E4" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="G4" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" s="1" t="b">
+      <c r="F4" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" s="1" t="b">
         <v>1</v>
       </c>
       <c r="J4" s="1" t="b">
@@ -2197,55 +2270,58 @@
       <c r="O4" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="1">
         <v>2</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="R4" s="1">
         <v>40</v>
       </c>
-      <c r="R4" s="1">
+      <c r="S4" s="1">
         <v>3</v>
       </c>
-      <c r="S4" s="1" t="str">
-        <f t="shared" ref="S4:S16" si="0">_xlfn.CONCAT("c(",P4,",",Q4,")")</f>
+      <c r="T4" s="1" t="str">
+        <f t="shared" ref="T4:T16" si="0">_xlfn.CONCAT("c(",Q4,",",R4,")")</f>
         <v>c(2,40)</v>
       </c>
-      <c r="T4" s="1">
-        <v>1</v>
-      </c>
       <c r="U4" s="1">
         <v>1</v>
       </c>
-      <c r="W4" s="1" t="s">
-        <v>122</v>
+      <c r="V4" s="1">
+        <v>1</v>
       </c>
       <c r="X4" s="1" t="s">
-        <v>127</v>
+        <v>185</v>
       </c>
       <c r="Y4" s="1" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="Z4" s="1" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="AA4" s="1" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.2">
+        <v>165</v>
+      </c>
+      <c r="AB4" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="AC4" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="5" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D5" s="1" t="b">
-        <v>1</v>
-      </c>
       <c r="E5" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="G5" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" s="1" t="b">
+      <c r="F5" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" s="1" t="b">
         <v>1</v>
       </c>
       <c r="J5" s="1" t="b">
@@ -2266,52 +2342,55 @@
       <c r="O5" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="P5" s="1">
+      <c r="P5" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q5" s="1">
         <v>2</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="R5" s="1">
         <v>40</v>
       </c>
-      <c r="R5" s="1">
+      <c r="S5" s="1">
         <v>3</v>
       </c>
-      <c r="S5" s="1" t="str">
+      <c r="T5" s="1" t="str">
         <f t="shared" si="0"/>
         <v>c(2,40)</v>
       </c>
-      <c r="T5" s="1">
-        <v>1</v>
-      </c>
       <c r="U5" s="1">
         <v>1</v>
       </c>
-      <c r="W5" s="1" t="s">
-        <v>123</v>
+      <c r="V5" s="1">
+        <v>1</v>
       </c>
       <c r="X5" s="1" t="s">
-        <v>128</v>
+        <v>185</v>
       </c>
       <c r="Y5" s="1" t="s">
-        <v>171</v>
+        <v>185</v>
       </c>
       <c r="Z5" s="1" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="AA5" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.2">
+        <v>166</v>
+      </c>
+      <c r="AB5" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="AC5" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="6" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D6" s="1" t="b">
-        <v>1</v>
-      </c>
       <c r="E6" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="I6" s="1" t="b">
+      <c r="F6" s="1" t="b">
         <v>1</v>
       </c>
       <c r="J6" s="1" t="b">
@@ -2332,42 +2411,48 @@
       <c r="O6" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="P6" s="1">
+      <c r="P6" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q6" s="1">
         <v>4</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="R6" s="1">
         <v>150</v>
       </c>
-      <c r="R6" s="1">
+      <c r="S6" s="1">
         <v>30</v>
       </c>
-      <c r="S6" s="1" t="str">
+      <c r="T6" s="1" t="str">
         <f t="shared" si="0"/>
         <v>c(4,150)</v>
       </c>
-      <c r="T6" s="1">
-        <v>1</v>
-      </c>
       <c r="U6" s="1">
         <v>1</v>
       </c>
-      <c r="W6" s="1" t="s">
-        <v>130</v>
+      <c r="V6" s="1">
+        <v>1</v>
       </c>
       <c r="X6" s="1" t="s">
-        <v>129</v>
+        <v>185</v>
       </c>
       <c r="Y6" s="1" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="Z6" s="1" t="s">
-        <v>141</v>
+        <v>126</v>
       </c>
       <c r="AA6" s="1" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.2">
+        <v>167</v>
+      </c>
+      <c r="AB6" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="AC6" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="7" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>41</v>
       </c>
@@ -2377,7 +2462,7 @@
       <c r="C7" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="H7" s="1" t="b">
+      <c r="D7" s="1" t="b">
         <v>1</v>
       </c>
       <c r="I7" s="1" t="b">
@@ -2401,45 +2486,51 @@
       <c r="O7" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="1">
         <v>2</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="R7" s="1">
         <v>150</v>
       </c>
-      <c r="R7" s="1">
+      <c r="S7" s="1">
         <v>20</v>
       </c>
-      <c r="S7" s="1" t="str">
+      <c r="T7" s="1" t="str">
         <f t="shared" si="0"/>
         <v>c(2,150)</v>
       </c>
-      <c r="T7" s="1">
-        <v>1</v>
-      </c>
       <c r="U7" s="1">
         <v>1</v>
       </c>
-      <c r="V7" s="1" t="s">
-        <v>118</v>
+      <c r="V7" s="1">
+        <v>1</v>
       </c>
       <c r="W7" s="1" t="s">
-        <v>132</v>
+        <v>117</v>
       </c>
       <c r="X7" s="1" t="s">
-        <v>133</v>
+        <v>128</v>
+      </c>
+      <c r="Y7" s="1" t="s">
+        <v>128</v>
       </c>
       <c r="Z7" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="AA7" s="1" t="s">
-        <v>142</v>
+        <v>129</v>
       </c>
       <c r="AB7" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="AC7" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="AD7" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="8" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>42</v>
       </c>
@@ -2449,7 +2540,7 @@
       <c r="C8" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="H8" s="1" t="b">
+      <c r="D8" s="1" t="b">
         <v>1</v>
       </c>
       <c r="I8" s="1" t="b">
@@ -2473,55 +2564,58 @@
       <c r="O8" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="1">
         <v>2</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="R8" s="1">
         <v>150</v>
       </c>
-      <c r="R8" s="1">
+      <c r="S8" s="1">
         <v>20</v>
       </c>
-      <c r="S8" s="1" t="str">
+      <c r="T8" s="1" t="str">
         <f t="shared" si="0"/>
         <v>c(2,150)</v>
       </c>
-      <c r="T8" s="1">
-        <v>1</v>
-      </c>
       <c r="U8" s="1">
         <v>1</v>
       </c>
-      <c r="V8" s="1" t="s">
-        <v>119</v>
+      <c r="V8" s="1">
+        <v>1</v>
       </c>
       <c r="W8" s="1" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="X8" s="1" t="s">
-        <v>134</v>
+        <v>127</v>
+      </c>
+      <c r="Y8" s="1" t="s">
+        <v>127</v>
       </c>
       <c r="Z8" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="AA8" s="1" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="AB8" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.2">
+        <v>139</v>
+      </c>
+      <c r="AC8" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="AD8" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="9" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="F9" s="1" t="b">
-        <v>1</v>
-      </c>
       <c r="G9" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="I9" s="1" t="b">
+      <c r="H9" s="1" t="b">
         <v>1</v>
       </c>
       <c r="J9" s="1" t="b">
@@ -2542,50 +2636,53 @@
       <c r="O9" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q9" s="1">
         <v>2</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="R9" s="1">
         <v>100</v>
       </c>
-      <c r="R9" s="1">
-        <f>P9+2</f>
+      <c r="S9" s="1">
+        <f>Q9+2</f>
         <v>4</v>
       </c>
-      <c r="S9" s="1" t="str">
+      <c r="T9" s="1" t="str">
         <f t="shared" si="0"/>
         <v>c(2,100)</v>
       </c>
-      <c r="T9" s="1">
-        <v>1</v>
-      </c>
       <c r="U9" s="1">
         <v>1</v>
       </c>
-      <c r="W9" s="1" t="s">
-        <v>135</v>
+      <c r="V9" s="1">
+        <v>1</v>
       </c>
       <c r="X9" s="1" t="s">
-        <v>135</v>
+        <v>185</v>
+      </c>
+      <c r="Y9" s="1" t="s">
+        <v>185</v>
       </c>
       <c r="Z9" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="AA9" s="1" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.2">
+        <v>131</v>
+      </c>
+      <c r="AB9" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="AC9" s="1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="10" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F10" s="1" t="b">
-        <v>1</v>
-      </c>
       <c r="G10" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="I10" s="1" t="b">
+      <c r="H10" s="1" t="b">
         <v>1</v>
       </c>
       <c r="J10" s="1" t="b">
@@ -2606,40 +2703,46 @@
       <c r="O10" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="1">
         <v>2</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="R10" s="1">
         <v>100</v>
       </c>
-      <c r="R10" s="1">
-        <f>P10+2</f>
+      <c r="S10" s="1">
+        <f>Q10+2</f>
         <v>4</v>
       </c>
-      <c r="S10" s="1" t="str">
+      <c r="T10" s="1" t="str">
         <f t="shared" si="0"/>
         <v>c(2,100)</v>
       </c>
-      <c r="T10" s="1">
-        <v>1</v>
-      </c>
       <c r="U10" s="1">
         <v>1</v>
       </c>
-      <c r="W10" s="1" t="s">
-        <v>136</v>
+      <c r="V10" s="1">
+        <v>1</v>
       </c>
       <c r="X10" s="1" t="s">
-        <v>136</v>
+        <v>185</v>
+      </c>
+      <c r="Y10" s="1" t="s">
+        <v>185</v>
       </c>
       <c r="Z10" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="AA10" s="1" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.2">
+        <v>132</v>
+      </c>
+      <c r="AB10" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="AC10" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="11" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>45</v>
       </c>
@@ -2658,7 +2761,7 @@
       <c r="G11" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="I11" s="1" t="b">
+      <c r="H11" s="1" t="b">
         <v>1</v>
       </c>
       <c r="J11" s="1" t="b">
@@ -2670,45 +2773,51 @@
       <c r="L11" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="O11" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="P11" s="1">
+      <c r="M11" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="P11" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q11" s="1">
         <v>0.01</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="R11" s="1">
         <v>0.2</v>
       </c>
-      <c r="R11" s="1">
+      <c r="S11" s="1">
         <v>0.1</v>
       </c>
-      <c r="S11" s="1" t="str">
+      <c r="T11" s="1" t="str">
         <f t="shared" si="0"/>
         <v>c(0.01,0.2)</v>
       </c>
-      <c r="T11" s="1">
-        <v>0.01</v>
-      </c>
       <c r="U11" s="1">
         <v>0.01</v>
       </c>
-      <c r="W11" s="1" t="s">
-        <v>124</v>
+      <c r="V11" s="1">
+        <v>0.01</v>
       </c>
       <c r="X11" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="Y11" s="1" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="Z11" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="AA11" s="1" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.2">
+        <v>168</v>
+      </c>
+      <c r="AB11" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="AC11" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="12" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>46</v>
       </c>
@@ -2724,123 +2833,126 @@
       <c r="E12" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="I12" s="1" t="b">
+      <c r="F12" s="1" t="b">
         <v>1</v>
       </c>
       <c r="J12" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="L12" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O12" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="P12" s="1">
+      <c r="K12" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="M12" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="P12" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q12" s="1">
         <v>0</v>
       </c>
-      <c r="Q12" s="1">
+      <c r="R12" s="1">
         <v>0.99</v>
       </c>
-      <c r="R12" s="1">
+      <c r="S12" s="1">
         <v>0.2</v>
       </c>
-      <c r="S12" s="1" t="str">
+      <c r="T12" s="1" t="str">
         <f t="shared" si="0"/>
         <v>c(0,0.99)</v>
       </c>
-      <c r="T12" s="1">
-        <v>0.01</v>
-      </c>
       <c r="U12" s="1">
         <v>0.01</v>
       </c>
-      <c r="V12" s="1" t="s">
-        <v>120</v>
+      <c r="V12" s="1">
+        <v>0.01</v>
       </c>
       <c r="W12" s="1" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="X12" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="Y12" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="Z12" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="AA12" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.2">
+        <v>122</v>
+      </c>
+      <c r="AB12" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="AC12" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="13" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>47</v>
       </c>
       <c r="C13" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="D13" s="1" t="b">
-        <v>1</v>
-      </c>
       <c r="E13" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="I13" s="1" t="b">
+      <c r="F13" s="1" t="b">
         <v>1</v>
       </c>
       <c r="J13" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="L13" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O13" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="P13" s="1">
+      <c r="K13" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="M13" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="P13" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q13" s="1">
         <v>0</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="R13" s="1">
         <v>0.99</v>
       </c>
-      <c r="R13" s="1">
+      <c r="S13" s="1">
         <v>0.2</v>
       </c>
-      <c r="S13" s="1" t="str">
+      <c r="T13" s="1" t="str">
         <f t="shared" si="0"/>
         <v>c(0,0.99)</v>
       </c>
-      <c r="T13" s="1">
-        <v>0.01</v>
-      </c>
       <c r="U13" s="1">
         <v>0.01</v>
       </c>
-      <c r="W13" s="1" t="s">
+      <c r="V13" s="1">
+        <v>0.01</v>
+      </c>
+      <c r="X13" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="X13" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="Y13" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="Z13" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="AA13" s="3" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="Z13" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="AA13" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="AB13" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="AC13" s="3" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="14" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="F14" s="1" t="b">
-        <v>1</v>
-      </c>
       <c r="G14" s="1" t="b">
         <v>1</v>
       </c>
@@ -2859,30 +2971,30 @@
       <c r="L14" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="O14" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="P14" s="1">
+      <c r="M14" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="P14" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q14" s="1">
         <v>0</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="R14" s="1">
         <v>0.99</v>
       </c>
-      <c r="R14" s="1">
+      <c r="S14" s="1">
         <v>0.25</v>
       </c>
-      <c r="S14" s="1" t="str">
+      <c r="T14" s="1" t="str">
         <f t="shared" si="0"/>
         <v>c(0,0.99)</v>
       </c>
-      <c r="T14" s="1">
-        <v>0.01</v>
-      </c>
       <c r="U14" s="1">
         <v>0.01</v>
       </c>
-      <c r="W14" s="1" t="s">
-        <v>49</v>
+      <c r="V14" s="1">
+        <v>0.01</v>
       </c>
       <c r="X14" s="1" t="s">
         <v>49</v>
@@ -2890,14 +3002,17 @@
       <c r="Z14" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="AA14" s="1" t="s">
+      <c r="AB14" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="AB14" s="1" t="s">
+      <c r="AC14" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AD14" s="1" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>50</v>
       </c>
@@ -2913,104 +3028,110 @@
       <c r="E15" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="I15" s="1" t="b">
+      <c r="F15" s="1" t="b">
         <v>1</v>
       </c>
       <c r="J15" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="L15" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="N15" s="1" t="b">
+      <c r="K15" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="M15" s="1" t="b">
         <v>1</v>
       </c>
       <c r="O15" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="1" t="b">
         <v>1</v>
       </c>
       <c r="Q15" s="1">
+        <v>1</v>
+      </c>
+      <c r="R15" s="1">
         <v>3</v>
       </c>
-      <c r="R15" s="1">
-        <v>1</v>
-      </c>
-      <c r="S15" s="1" t="str">
+      <c r="S15" s="1">
+        <v>1</v>
+      </c>
+      <c r="T15" s="1" t="str">
         <f t="shared" si="0"/>
         <v>c(1,3)</v>
       </c>
-      <c r="T15" s="1">
-        <v>1</v>
-      </c>
       <c r="U15" s="1">
         <v>1</v>
       </c>
-      <c r="V15" s="1" t="s">
+      <c r="V15" s="1">
+        <v>1</v>
+      </c>
+      <c r="W15" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="W15" s="1" t="s">
-        <v>139</v>
-      </c>
       <c r="X15" s="1" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="Y15" s="1" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="Z15" s="1" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="AA15" s="1" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+      <c r="AB15" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="AC15" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="16" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="C16" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="J16" s="1" t="b">
-        <v>1</v>
-      </c>
       <c r="K16" s="1" t="b">
         <v>1</v>
       </c>
       <c r="L16" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="O16" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="P16" s="1">
+      <c r="M16" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="P16" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q16" s="1">
         <v>0.01</v>
       </c>
-      <c r="Q16" s="1">
+      <c r="R16" s="1">
         <v>3.25</v>
       </c>
-      <c r="R16" s="1">
+      <c r="S16" s="1">
         <v>0.15</v>
       </c>
-      <c r="S16" s="1" t="str">
+      <c r="T16" s="1" t="str">
         <f t="shared" si="0"/>
         <v>c(0.01,3.25)</v>
       </c>
-      <c r="T16" s="1">
-        <v>0.01</v>
-      </c>
       <c r="U16" s="1">
         <v>0.01</v>
       </c>
-      <c r="W16" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="Z16" s="1" t="s">
+      <c r="V16" s="1">
+        <v>0.01</v>
+      </c>
+      <c r="X16" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="AB16" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="AA16" s="1" t="s">
+      <c r="AC16" s="1" t="s">
         <v>53</v>
       </c>
     </row>
@@ -3023,7 +3144,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D24D9501-1928-C24A-A5F8-EF63F20DDAEF}">
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.33203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="33.5" style="4" bestFit="1" customWidth="1"/>
@@ -3044,7 +3165,7 @@
         <v>55</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>56</v>
@@ -3055,7 +3176,7 @@
         <v>57</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>58</v>
@@ -3066,16 +3187,16 @@
         <v>59</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>60</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -3083,7 +3204,7 @@
         <v>61</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>56</v>
@@ -3094,7 +3215,7 @@
         <v>62</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>63</v>
@@ -3105,16 +3226,16 @@
         <v>64</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>60</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -3122,7 +3243,7 @@
         <v>65</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>66</v>
@@ -3133,10 +3254,10 @@
         <v>67</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
@@ -3144,16 +3265,16 @@
         <v>68</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>60</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
@@ -3161,7 +3282,7 @@
         <v>69</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>66</v>
@@ -3172,10 +3293,10 @@
         <v>70</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
@@ -3183,16 +3304,16 @@
         <v>71</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>60</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
@@ -3200,7 +3321,7 @@
         <v>72</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>66</v>
@@ -3211,10 +3332,10 @@
         <v>73</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
@@ -3222,16 +3343,16 @@
         <v>74</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>60</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
@@ -3239,7 +3360,7 @@
         <v>75</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>66</v>
@@ -3250,10 +3371,10 @@
         <v>76</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -3261,52 +3382,52 @@
         <v>77</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>60</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
-        <v>78</v>
+        <v>187</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
-        <v>80</v>
+        <v>188</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>81</v>
+        <v>152</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
-        <v>82</v>
+        <v>189</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="E22" s="5" t="s">
         <v>158</v>
@@ -3314,181 +3435,259 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
-        <v>84</v>
+        <v>190</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
-        <v>85</v>
+        <v>191</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
-        <v>86</v>
+        <v>192</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>159</v>
+        <v>193</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
-        <v>175</v>
+        <v>78</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>182</v>
+        <v>79</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
-        <v>176</v>
+        <v>80</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>181</v>
+        <v>81</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
-        <v>177</v>
+        <v>82</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>83</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>183</v>
+        <v>154</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
-        <v>178</v>
+        <v>84</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>182</v>
+        <v>79</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
-        <v>179</v>
+        <v>85</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>184</v>
+        <v>150</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
-        <v>180</v>
+        <v>86</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>83</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>185</v>
+        <v>155</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A33" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A35" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="E37" s="5" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B32" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="C32" s="5" t="s">
+      <c r="B38" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="C38" s="5" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A33" s="4" t="s">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="B33" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="C33" s="5" t="s">
+      <c r="B39" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="C39" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A34" s="4" t="s">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A40" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B34" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="C34" s="5" t="s">
+      <c r="B40" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="C40" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A35" s="4" t="s">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A41" s="4" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A36" s="4" t="s">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A42" s="4" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A37" s="4" t="s">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A43" s="4" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A38" s="4" t="s">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A44" s="4" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A39" s="4" t="s">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A45" s="4" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A40" s="4" t="s">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A46" s="4" t="s">
         <v>92</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated for july 2022
</commit_message>
<xml_diff>
--- a/support materials/menuManager.xlsx
+++ b/support materials/menuManager.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10711"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hedbergec/Dropbox/Papers/Paper.QEDs/Apps/plannerApp/support materials/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hedbe\Dropbox\Papers\Paper.QEDs\Apps\plannerApp\support materials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B00D196E-A740-BA45-A476-247132802E46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58BD68F8-3966-4D7A-9E9B-A328CF4646A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16260" tabRatio="716" activeTab="6" xr2:uid="{8D89E9AD-B3C8-4CE6-A909-5B9DBA95DCBB}"/>
+    <workbookView xWindow="1103" yWindow="1103" windowWidth="16875" windowHeight="10575" tabRatio="716" activeTab="6" xr2:uid="{8D89E9AD-B3C8-4CE6-A909-5B9DBA95DCBB}"/>
   </bookViews>
   <sheets>
     <sheet name="readme" sheetId="11" r:id="rId1"/>
@@ -1445,22 +1445,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C51C3392-495A-4716-B7D0-8CB1570246E2}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="21.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="str">
         <f>HYPERLINK(sample!A1)</f>
         <v>sample</v>
@@ -1469,7 +1469,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="str">
         <f>HYPERLINK(design!A1)</f>
         <v>design</v>
@@ -1478,7 +1478,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="str">
         <f>HYPERLINK(inference!A1)</f>
         <v>inference</v>
@@ -1487,7 +1487,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="str">
         <f>HYPERLINK(model!A1)</f>
         <v>model</v>
@@ -1496,7 +1496,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="str">
         <f>HYPERLINK(stat!A1)</f>
         <v>stat</v>
@@ -1505,7 +1505,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" s="2" t="str">
         <f>HYPERLINK(input!A1)</f>
         <v>input</v>
@@ -1514,13 +1514,13 @@
         <v>110</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" s="2"/>
       <c r="C9" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" s="2" t="str">
         <f>HYPERLINK(code!A1,"code")</f>
         <v>code</v>
@@ -1529,7 +1529,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="C11" t="s">
         <v>108</v>
       </c>
@@ -1542,9 +1542,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A96E0447-8401-42C5-BE02-401F505AE938}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1552,7 +1552,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1560,7 +1560,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1576,12 +1576,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62AA0D0E-E4D1-469A-AF1F-085E17D5518F}">
   <dimension ref="A1:D9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="29.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -1595,7 +1595,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1606,7 +1606,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>176</v>
       </c>
@@ -1617,7 +1617,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1628,7 +1628,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1639,7 +1639,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>162</v>
       </c>
@@ -1650,7 +1650,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -1661,7 +1661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -1672,7 +1672,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>93</v>
       </c>
@@ -1691,13 +1691,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33C6AD60-7AB8-4CAF-9726-0F1707E818DE}">
   <dimension ref="A1:J3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="5.1640625" customWidth="1"/>
+    <col min="3" max="4" width="5.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -1729,7 +1729,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -1755,7 +1755,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1777,14 +1777,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F39838A5-C062-40CB-BD39-4466E5E1974A}">
   <dimension ref="A1:J3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.1328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="5.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -1816,7 +1816,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -1848,7 +1848,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -1879,13 +1879,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9306200-6D5D-404E-9AA4-2D83AC7E89FD}">
   <dimension ref="A1:J4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="22.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>20</v>
       </c>
@@ -1917,7 +1917,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -1949,7 +1949,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -1981,7 +1981,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -2022,20 +2022,20 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7085B87C-0BDF-4509-A80F-252767BE3B26}">
   <dimension ref="A1:AD17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" style="1" customWidth="1"/>
     <col min="3" max="4" width="8" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.1328125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="8" width="5.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="5.33203125" style="1" customWidth="1"/>
-    <col min="10" max="11" width="7.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="7.796875" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="16" width="7.83203125" style="1" customWidth="1"/>
-    <col min="17" max="18" width="9.1640625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="9.1328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="16" width="7.796875" style="1" customWidth="1"/>
+    <col min="17" max="18" width="9.1328125" style="1" customWidth="1"/>
     <col min="19" max="19" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="14.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="21" max="22" width="14.6640625" style="1" customWidth="1"/>
@@ -2044,10 +2044,10 @@
     <col min="26" max="26" width="49.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="49.33203125" style="1" customWidth="1"/>
     <col min="28" max="29" width="55.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="16384" width="9.1640625" style="1"/>
+    <col min="30" max="16384" width="9.1328125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>27</v>
       </c>
@@ -2139,7 +2139,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>37</v>
       </c>
@@ -2214,7 +2214,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>38</v>
       </c>
@@ -2280,7 +2280,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>39</v>
       </c>
@@ -2346,7 +2346,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>190</v>
       </c>
@@ -2394,7 +2394,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>191</v>
       </c>
@@ -2442,7 +2442,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>40</v>
       </c>
@@ -2474,7 +2474,7 @@
         <v>1</v>
       </c>
       <c r="Q7" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R7" s="1">
         <v>150</v>
@@ -2484,13 +2484,13 @@
       </c>
       <c r="T7" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>c(4,150)</v>
+        <v>c(5,150)</v>
       </c>
       <c r="U7" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="V7" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="X7" s="1" t="s">
         <v>178</v>
@@ -2511,7 +2511,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>41</v>
       </c>
@@ -2549,23 +2549,23 @@
         <v>1</v>
       </c>
       <c r="Q8" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R8" s="1">
-        <v>150</v>
+        <v>500</v>
       </c>
       <c r="S8" s="1">
         <v>20</v>
       </c>
       <c r="T8" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>c(2,150)</v>
+        <v>c(5,500)</v>
       </c>
       <c r="U8" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="V8" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="W8" s="1" t="s">
         <v>117</v>
@@ -2589,7 +2589,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>42</v>
       </c>
@@ -2627,23 +2627,23 @@
         <v>1</v>
       </c>
       <c r="Q9" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R9" s="1">
-        <v>150</v>
+        <v>500</v>
       </c>
       <c r="S9" s="1">
         <v>20</v>
       </c>
       <c r="T9" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>c(2,150)</v>
+        <v>c(5,500)</v>
       </c>
       <c r="U9" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="V9" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="W9" s="1" t="s">
         <v>118</v>
@@ -2667,7 +2667,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>43</v>
       </c>
@@ -2734,7 +2734,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>44</v>
       </c>
@@ -2801,7 +2801,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>45</v>
       </c>
@@ -2876,7 +2876,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>46</v>
       </c>
@@ -2948,7 +2948,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>47</v>
       </c>
@@ -3008,7 +3008,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>48</v>
       </c>
@@ -3071,7 +3071,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>50</v>
       </c>
@@ -3146,7 +3146,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="17" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
         <v>145</v>
       </c>
@@ -3204,22 +3204,22 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D24D9501-1928-C24A-A5F8-EF63F20DDAEF}">
   <dimension ref="A1:E46"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.33203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.33203125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="33.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="33.5" style="4" customWidth="1"/>
-    <col min="3" max="3" width="42.1640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5" style="5" customWidth="1"/>
+    <col min="1" max="1" width="33.46484375" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.46484375" style="4" customWidth="1"/>
+    <col min="3" max="3" width="42.1328125" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.46484375" style="5" customWidth="1"/>
     <col min="5" max="5" width="92.6640625" style="5" bestFit="1" customWidth="1"/>
     <col min="6" max="16384" width="11.33203125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" s="4" t="s">
         <v>55</v>
       </c>
@@ -3230,7 +3230,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" s="4" t="s">
         <v>57</v>
       </c>
@@ -3241,7 +3241,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" s="4" t="s">
         <v>59</v>
       </c>
@@ -3258,7 +3258,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" s="4" t="s">
         <v>61</v>
       </c>
@@ -3269,7 +3269,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
         <v>62</v>
       </c>
@@ -3280,7 +3280,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
         <v>64</v>
       </c>
@@ -3297,7 +3297,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" s="4" t="s">
         <v>65</v>
       </c>
@@ -3308,7 +3308,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9" s="4" t="s">
         <v>67</v>
       </c>
@@ -3319,7 +3319,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A10" s="4" t="s">
         <v>68</v>
       </c>
@@ -3336,7 +3336,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" s="4" t="s">
         <v>69</v>
       </c>
@@ -3347,7 +3347,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" s="4" t="s">
         <v>70</v>
       </c>
@@ -3358,7 +3358,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A13" s="4" t="s">
         <v>71</v>
       </c>
@@ -3375,7 +3375,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A14" s="4" t="s">
         <v>72</v>
       </c>
@@ -3386,7 +3386,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A15" s="4" t="s">
         <v>73</v>
       </c>
@@ -3397,7 +3397,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A16" s="4" t="s">
         <v>74</v>
       </c>
@@ -3414,7 +3414,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17" s="4" t="s">
         <v>75</v>
       </c>
@@ -3425,7 +3425,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A18" s="4" t="s">
         <v>76</v>
       </c>
@@ -3436,7 +3436,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A19" s="4" t="s">
         <v>77</v>
       </c>
@@ -3453,7 +3453,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A20" s="4" t="s">
         <v>180</v>
       </c>
@@ -3464,7 +3464,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A21" s="4" t="s">
         <v>181</v>
       </c>
@@ -3475,7 +3475,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A22" s="4" t="s">
         <v>182</v>
       </c>
@@ -3492,7 +3492,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A23" s="4" t="s">
         <v>183</v>
       </c>
@@ -3503,7 +3503,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A24" s="4" t="s">
         <v>184</v>
       </c>
@@ -3514,7 +3514,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A25" s="4" t="s">
         <v>185</v>
       </c>
@@ -3531,7 +3531,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A26" s="4" t="s">
         <v>78</v>
       </c>
@@ -3542,7 +3542,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A27" s="4" t="s">
         <v>80</v>
       </c>
@@ -3553,7 +3553,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A28" s="4" t="s">
         <v>82</v>
       </c>
@@ -3570,7 +3570,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A29" s="4" t="s">
         <v>84</v>
       </c>
@@ -3581,7 +3581,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A30" s="4" t="s">
         <v>85</v>
       </c>
@@ -3592,7 +3592,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A31" s="4" t="s">
         <v>86</v>
       </c>
@@ -3609,7 +3609,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A32" s="4" t="s">
         <v>169</v>
       </c>
@@ -3620,7 +3620,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A33" s="4" t="s">
         <v>170</v>
       </c>
@@ -3631,7 +3631,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A34" s="4" t="s">
         <v>171</v>
       </c>
@@ -3648,7 +3648,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A35" s="4" t="s">
         <v>172</v>
       </c>
@@ -3659,7 +3659,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A36" s="4" t="s">
         <v>173</v>
       </c>
@@ -3670,7 +3670,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A37" s="4" t="s">
         <v>174</v>
       </c>
@@ -3687,7 +3687,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A38" s="4" t="s">
         <v>96</v>
       </c>
@@ -3698,7 +3698,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A39" s="4" t="s">
         <v>97</v>
       </c>
@@ -3709,7 +3709,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A40" s="4" t="s">
         <v>98</v>
       </c>
@@ -3720,32 +3720,32 @@
         <v>99</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A41" s="4" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A42" s="4" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A43" s="4" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A44" s="4" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A45" s="4" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A46" s="4" t="s">
         <v>92</v>
       </c>

</xml_diff>